<commit_message>
feat: import scripts for all 13 templates, de/en representatives imported; parser fixes (accordion links, span text)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="100">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,114 @@
     <t>url</t>
   </si>
   <si>
+    <t>de/en/100-years.report.json</t>
+  </si>
+  <si>
+    <t>["hero-campaign","hero-campaign","columns-media","columns-media","columns-media","columns-media","cards-teaser","cards-teaser"]</t>
+  </si>
+  <si>
+    <t>de/en/100-years</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>campaign</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:07.829Z</t>
+  </si>
+  <si>
+    <t>100 Years Lufthansa | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/100-years</t>
+  </si>
+  <si>
+    <t>de/en/359.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-lightbox","table-striped"]</t>
+  </si>
+  <si>
+    <t>de/en/359</t>
+  </si>
+  <si>
+    <t>fleet</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:12.414Z</t>
+  </si>
+  <si>
+    <t>Airbus A350-900 | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/359</t>
+  </si>
+  <si>
+    <t>de/en/baggage.report.json</t>
+  </si>
+  <si>
+    <t>["cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","columns-media"]</t>
+  </si>
+  <si>
+    <t>de/en/baggage</t>
+  </si>
+  <si>
+    <t>hub</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:54:59.566Z</t>
+  </si>
+  <si>
+    <t>Baggage | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/baggage</t>
+  </si>
+  <si>
+    <t>de/en/feedback.report.json</t>
+  </si>
+  <si>
+    <t>["form","accordion-columns"]</t>
+  </si>
+  <si>
+    <t>de/en/feedback</t>
+  </si>
+  <si>
+    <t>form</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:25.934Z</t>
+  </si>
+  <si>
+    <t>Feedback and other contact forms | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/feedback</t>
+  </si>
+  <si>
+    <t>de/en/flying-with-small-children.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-columns","carousel-cards"]</t>
+  </si>
+  <si>
+    <t>de/en/flying-with-small-children</t>
+  </si>
+  <si>
+    <t>info</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:03.691Z</t>
+  </si>
+  <si>
+    <t>Flying with small children | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/flying-with-small-children</t>
+  </si>
+  <si>
     <t>de/en/homepage.report.json</t>
   </si>
   <si>
@@ -46,19 +154,163 @@
     <t>de/en/homepage</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-21T14:41:22.080Z</t>
+    <t>2026-10-21T17:01:12.172Z</t>
   </si>
   <si>
     <t>Book your flight now - travel with Lufthansa to over 200 destinations | Lufthansa</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/homepage</t>
+  </si>
+  <si>
+    <t>de/en/imprint.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>de/en/imprint</t>
+  </si>
+  <si>
+    <t>legal</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:21.743Z</t>
+  </si>
+  <si>
+    <t>Legal notice | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/imprint</t>
+  </si>
+  <si>
+    <t>de/en/online-check-in.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","cards-steps","booking-lookup","cards-teaser"]</t>
+  </si>
+  <si>
+    <t>de/en/online-check-in</t>
+  </si>
+  <si>
+    <t>app-entry</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:30.108Z</t>
+  </si>
+  <si>
+    <t>Online check-in | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/online-check-in</t>
+  </si>
+  <si>
+    <t>de/en/timetable-and-flight-status.report.json</t>
+  </si>
+  <si>
+    <t>["flight-status","columns-media","columns-media","columns-media","accordion-columns"]</t>
+  </si>
+  <si>
+    <t>de/en/timetable-and-flight-status</t>
+  </si>
+  <si>
+    <t>flight-status</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:35.097Z</t>
+  </si>
+  <si>
+    <t>Timetable &amp; flight status | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/timetable-and-flight-status</t>
+  </si>
+  <si>
+    <t>lhg/de/en.report.json</t>
+  </si>
+  <si>
+    <t>["flight-search","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price","cards-price"]</t>
+  </si>
+  <si>
+    <t>lhg/de/en</t>
+  </si>
+  <si>
+    <t>aircore-destination-overview</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:43.571Z</t>
+  </si>
+  <si>
+    <t>Book flights to destinations all over the world | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/lhg/de/en</t>
+  </si>
+  <si>
+    <t>de/en/articles/explore-the-world/eat-see-do-berlin.report.json</t>
+  </si>
+  <si>
+    <t>["article-header","price-bar","carousel-cards","columns-media","related-articles"]</t>
+  </si>
+  <si>
+    <t>de/en/articles/explore-the-world/eat-see-do-berlin</t>
+  </si>
+  <si>
+    <t>insights</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:17.564Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/articles/explore-the-world/eat-see-do-berlin</t>
+  </si>
+  <si>
+    <t>lhg/de/en/dest/cy/new-york.report.json</t>
+  </si>
+  <si>
+    <t>["flight-search","cards-price","accordion-columns","accordion-columns","table-deals","cards-icon-text","weather","accordion-side-by-side"]</t>
+  </si>
+  <si>
+    <t>lhg/de/en/dest/cy/new-york</t>
+  </si>
+  <si>
+    <t>aircore-destination</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:48.147Z</t>
+  </si>
+  <si>
+    <t>Flight to New York (NYC) | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/lhg/de/en/dest/cy/new-york</t>
+  </si>
+  <si>
+    <t>lhg/de/en/o-d/c-c/germany-usa.report.json</t>
+  </si>
+  <si>
+    <t>["flight-search","cards-icon-text","accordion-columns","accordion-side-by-side"]</t>
+  </si>
+  <si>
+    <t>lhg/de/en/o-d/c-c/germany-usa</t>
+  </si>
+  <si>
+    <t>aircore-route</t>
+  </si>
+  <si>
+    <t>2026-10-21T16:55:53.415Z</t>
+  </si>
+  <si>
+    <t>Flights from Germany to USA | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/lhg/de/en/o-d/c-c/germany-usa</t>
   </si>
 </sst>
 </file>
@@ -447,16 +699,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="42" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +758,318 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" t="s">
+        <v>91</v>
+      </c>
+      <c r="H13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" t="s">
+        <v>97</v>
+      </c>
+      <c r="G14" t="s">
+        <v>98</v>
+      </c>
+      <c r="H14" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: DA upload + preview tool (scope-limited, preview only); homepages for de/de, at/de, gb/en imported; onboard pages first in capture queue
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="171">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,9 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>fragment</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -37,6 +40,99 @@
     <t>url</t>
   </si>
   <si>
+    <t>at/de/footer.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>footer</t>
+  </si>
+  <si>
+    <t>at/de/footer</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>nav</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:55:06.747Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/at/de/homepage#footer</t>
+  </si>
+  <si>
+    <t>at/de/homepage.report.json</t>
+  </si>
+  <si>
+    <t>["flight-search","hero-card-overlay","fare-teaser","carousel-cards","destination-finder","cards-icon","columns-logos","accordion-columns"]</t>
+  </si>
+  <si>
+    <t>at/de/homepage</t>
+  </si>
+  <si>
+    <t>homepage</t>
+  </si>
+  <si>
+    <t>2026-10-21T18:23:02.162Z</t>
+  </si>
+  <si>
+    <t>Jetzt Flug buchen – mit Lufthansa zu über 200 Zielen reisen | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/at/de/homepage</t>
+  </si>
+  <si>
+    <t>at/de/nav.report.json</t>
+  </si>
+  <si>
+    <t>at/de/nav</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:55:02.759Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/at/de/homepage#nav</t>
+  </si>
+  <si>
+    <t>de/de/footer.report.json</t>
+  </si>
+  <si>
+    <t>de/de/footer</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:54:56.409Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/de/homepage#footer</t>
+  </si>
+  <si>
+    <t>de/de/homepage.report.json</t>
+  </si>
+  <si>
+    <t>de/de/homepage</t>
+  </si>
+  <si>
+    <t>2026-10-21T18:22:56.557Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/de/homepage</t>
+  </si>
+  <si>
+    <t>de/de/nav.report.json</t>
+  </si>
+  <si>
+    <t>de/de/nav</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:54:52.930Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/de/homepage#nav</t>
+  </si>
+  <si>
     <t>de/en/100-years.report.json</t>
   </si>
   <si>
@@ -46,9 +142,6 @@
     <t>de/en/100-years</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>campaign</t>
   </si>
   <si>
@@ -115,7 +208,7 @@
     <t>form</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:25.934Z</t>
+    <t>2026-10-21T17:01:26.038Z</t>
   </si>
   <si>
     <t>Feedback and other contact forms | Lufthansa</t>
@@ -136,7 +229,7 @@
     <t>info</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:03.691Z</t>
+    <t>2026-10-21T17:01:18.757Z</t>
   </si>
   <si>
     <t>Flying with small children | Lufthansa</t>
@@ -145,18 +238,24 @@
     <t>https://www.lufthansa.com/de/en/flying-with-small-children</t>
   </si>
   <si>
+    <t>de/en/footer.report.json</t>
+  </si>
+  <si>
+    <t>de/en/footer</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:54:45.381Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/homepage#footer</t>
+  </si>
+  <si>
     <t>de/en/homepage.report.json</t>
   </si>
   <si>
-    <t>["flight-search","hero-card-overlay","fare-teaser","carousel-cards","destination-finder","cards-icon","columns-logos","accordion-columns"]</t>
-  </si>
-  <si>
     <t>de/en/homepage</t>
   </si>
   <si>
-    <t>homepage</t>
-  </si>
-  <si>
     <t>2026-10-21T17:01:12.172Z</t>
   </si>
   <si>
@@ -187,6 +286,18 @@
     <t>https://www.lufthansa.com/de/en/imprint</t>
   </si>
   <si>
+    <t>de/en/nav.report.json</t>
+  </si>
+  <si>
+    <t>de/en/nav</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:54:40.832Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/homepage#nav</t>
+  </si>
+  <si>
     <t>de/en/online-check-in.report.json</t>
   </si>
   <si>
@@ -220,7 +331,7 @@
     <t>flight-status</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:35.097Z</t>
+    <t>2026-10-21T17:01:33.445Z</t>
   </si>
   <si>
     <t>Timetable &amp; flight status | Lufthansa</t>
@@ -229,6 +340,42 @@
     <t>https://www.lufthansa.com/de/en/timetable-and-flight-status</t>
   </si>
   <si>
+    <t>gb/en/footer.report.json</t>
+  </si>
+  <si>
+    <t>gb/en/footer</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:55:19.112Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/gb/en/homepage#footer</t>
+  </si>
+  <si>
+    <t>gb/en/homepage.report.json</t>
+  </si>
+  <si>
+    <t>gb/en/homepage</t>
+  </si>
+  <si>
+    <t>2026-10-21T18:23:07.976Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/gb/en/homepage</t>
+  </si>
+  <si>
+    <t>gb/en/nav.report.json</t>
+  </si>
+  <si>
+    <t>gb/en/nav</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:55:14.658Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/gb/en/homepage#nav</t>
+  </si>
+  <si>
     <t>lhg/de/en.report.json</t>
   </si>
   <si>
@@ -250,6 +397,78 @@
     <t>https://www.lufthansa.com/lhg/de/en</t>
   </si>
   <si>
+    <t>at/de/fragments/payment-social.report.json</t>
+  </si>
+  <si>
+    <t>payment-social</t>
+  </si>
+  <si>
+    <t>at/de/fragments/payment-social</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:55:10.878Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/at/de/homepage#payment-social</t>
+  </si>
+  <si>
+    <t>de/de/fragments/payment-social.report.json</t>
+  </si>
+  <si>
+    <t>de/de/fragments/payment-social</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:54:59.638Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/de/homepage#payment-social</t>
+  </si>
+  <si>
+    <t>de/en/fragments/payment-social.report.json</t>
+  </si>
+  <si>
+    <t>de/en/fragments/payment-social</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:54:49.651Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/homepage#payment-social</t>
+  </si>
+  <si>
+    <t>gb/en/fragments/payment-social.report.json</t>
+  </si>
+  <si>
+    <t>gb/en/fragments/payment-social</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:55:24.929Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/gb/en/homepage#payment-social</t>
+  </si>
+  <si>
+    <t>lhg/de/en/zz-test.report.json</t>
+  </si>
+  <si>
+    <t>["cards-icon-text"]</t>
+  </si>
+  <si>
+    <t>lhg/de/en/zz-test</t>
+  </si>
+  <si>
+    <t>aircore-destination</t>
+  </si>
+  <si>
+    <t>2026-10-21T17:04:36.900Z</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/lhg/de/en/zz-test</t>
+  </si>
+  <si>
     <t>de/en/articles/explore-the-world/eat-see-do-berlin.report.json</t>
   </si>
   <si>
@@ -265,9 +484,6 @@
     <t>2026-10-21T16:55:17.564Z</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>https://www.lufthansa.com/de/en/articles/explore-the-world/eat-see-do-berlin</t>
   </si>
   <si>
@@ -280,10 +496,7 @@
     <t>lhg/de/en/dest/cy/new-york</t>
   </si>
   <si>
-    <t>aircore-destination</t>
-  </si>
-  <si>
-    <t>2026-10-21T16:55:48.147Z</t>
+    <t>2026-10-21T17:07:20.550Z</t>
   </si>
   <si>
     <t>Flight to New York (NYC) | Lufthansa</t>
@@ -304,7 +517,7 @@
     <t>aircore-route</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:53.415Z</t>
+    <t>2026-10-21T17:07:24.799Z</t>
   </si>
   <si>
     <t>Flights from Germany to USA | Lufthansa</t>
@@ -699,16 +912,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="50" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="8" width="50" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -733,48 +948,54 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
         <v>20</v>
@@ -785,295 +1006,795 @@
       <c r="H3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="E4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="D5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" t="s">
+      <c r="H5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" t="s">
         <v>11</v>
       </c>
-      <c r="E5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="D13" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>77</v>
+      </c>
+      <c r="H13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" t="s">
+        <v>82</v>
+      </c>
+      <c r="I14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
+        <v>88</v>
+      </c>
+      <c r="H15" t="s">
+        <v>89</v>
+      </c>
+      <c r="I15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>93</v>
+      </c>
+      <c r="H16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I16" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" t="s">
+        <v>99</v>
+      </c>
+      <c r="H17" t="s">
+        <v>100</v>
+      </c>
+      <c r="I17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G18" t="s">
+        <v>106</v>
+      </c>
+      <c r="H18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" t="s">
         <v>11</v>
       </c>
-      <c r="E6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" t="s">
-        <v>41</v>
-      </c>
-      <c r="G6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" t="s">
-        <v>56</v>
-      </c>
-      <c r="H8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>61</v>
-      </c>
-      <c r="F9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" t="s">
-        <v>63</v>
-      </c>
-      <c r="H9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" t="s">
-        <v>67</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>68</v>
-      </c>
-      <c r="F10" t="s">
-        <v>69</v>
-      </c>
-      <c r="G10" t="s">
-        <v>70</v>
-      </c>
-      <c r="H10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>72</v>
-      </c>
-      <c r="B11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C11" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>75</v>
-      </c>
-      <c r="F11" t="s">
-        <v>76</v>
-      </c>
-      <c r="G11" t="s">
-        <v>77</v>
-      </c>
-      <c r="H11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" t="s">
-        <v>80</v>
-      </c>
-      <c r="C12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="D19" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>111</v>
+      </c>
+      <c r="H19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
+        <v>114</v>
+      </c>
+      <c r="E20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" t="s">
+        <v>115</v>
+      </c>
+      <c r="H20" t="s">
         <v>82</v>
       </c>
-      <c r="F12" t="s">
-        <v>83</v>
-      </c>
-      <c r="G12" t="s">
-        <v>84</v>
-      </c>
-      <c r="H12" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" t="s">
-        <v>88</v>
-      </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>89</v>
-      </c>
-      <c r="F13" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" t="s">
-        <v>91</v>
-      </c>
-      <c r="H13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C14" t="s">
-        <v>95</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>96</v>
-      </c>
-      <c r="F14" t="s">
-        <v>97</v>
-      </c>
-      <c r="G14" t="s">
-        <v>98</v>
-      </c>
-      <c r="H14" t="s">
-        <v>99</v>
+      <c r="I20" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>119</v>
+      </c>
+      <c r="H21" t="s">
+        <v>10</v>
+      </c>
+      <c r="I21" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" t="s">
+        <v>123</v>
+      </c>
+      <c r="E22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" t="s">
+        <v>124</v>
+      </c>
+      <c r="G22" t="s">
+        <v>125</v>
+      </c>
+      <c r="H22" t="s">
+        <v>126</v>
+      </c>
+      <c r="I22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" t="s">
+        <v>129</v>
+      </c>
+      <c r="D23" t="s">
+        <v>130</v>
+      </c>
+      <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>131</v>
+      </c>
+      <c r="H23" t="s">
+        <v>10</v>
+      </c>
+      <c r="I23" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>135</v>
+      </c>
+      <c r="H24" t="s">
+        <v>10</v>
+      </c>
+      <c r="I24" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>137</v>
+      </c>
+      <c r="B25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>129</v>
+      </c>
+      <c r="D25" t="s">
+        <v>138</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>139</v>
+      </c>
+      <c r="H25" t="s">
+        <v>10</v>
+      </c>
+      <c r="I25" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" t="s">
+        <v>142</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>143</v>
+      </c>
+      <c r="H26" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>145</v>
+      </c>
+      <c r="B27" t="s">
+        <v>146</v>
+      </c>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" t="s">
+        <v>147</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
+        <v>148</v>
+      </c>
+      <c r="G27" t="s">
+        <v>149</v>
+      </c>
+      <c r="H27" t="s">
+        <v>150</v>
+      </c>
+      <c r="I27" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>152</v>
+      </c>
+      <c r="B28" t="s">
+        <v>153</v>
+      </c>
+      <c r="C28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" t="s">
+        <v>154</v>
+      </c>
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" t="s">
+        <v>155</v>
+      </c>
+      <c r="G28" t="s">
+        <v>156</v>
+      </c>
+      <c r="H28" t="s">
+        <v>10</v>
+      </c>
+      <c r="I28" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>158</v>
+      </c>
+      <c r="B29" t="s">
+        <v>159</v>
+      </c>
+      <c r="C29" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" t="s">
+        <v>160</v>
+      </c>
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" t="s">
+        <v>148</v>
+      </c>
+      <c r="G29" t="s">
+        <v>161</v>
+      </c>
+      <c r="H29" t="s">
+        <v>162</v>
+      </c>
+      <c r="I29" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>164</v>
+      </c>
+      <c r="B30" t="s">
+        <v>165</v>
+      </c>
+      <c r="C30" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" t="s">
+        <v>166</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
+        <v>167</v>
+      </c>
+      <c r="G30" t="s">
+        <v>168</v>
+      </c>
+      <c r="H30" t="s">
+        <v>169</v>
+      </c>
+      <c r="I30" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: importer media limits (SVG>40KB rasterized, images <=2560px, long lists split into fragments), destination-finder grid, breadcrumb block; direct live calls for suggestions/labels/catalogs/defaultAirport with recorded fallback, data-lh-source; UI recorder removed
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1737" uniqueCount="996">
   <si>
     <t>_reportFile</t>
   </si>
@@ -76,7 +76,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-21T22:28:43.065Z</t>
+    <t>2026-10-22T00:04:34.822Z</t>
   </si>
   <si>
     <t>Jetzt Flug buchen – mit Lufthansa zu über 200 Zielen reisen | Lufthansa</t>
@@ -109,7 +109,7 @@
     <t>info</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:02.890Z</t>
+    <t>2026-10-21T22:32:06.345Z</t>
   </si>
   <si>
     <t>Doctor on Board – Gut zu wissen | Lufthansa</t>
@@ -127,7 +127,7 @@
     <t>de/de/doctor-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:59.676Z</t>
+    <t>2026-10-21T22:32:01.082Z</t>
   </si>
   <si>
     <t>Doctor on Board | Lufthansa</t>
@@ -154,7 +154,7 @@
     <t>de/de/homepage</t>
   </si>
   <si>
-    <t>2026-10-21T22:28:39.550Z</t>
+    <t>2026-10-22T00:04:31.566Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/homepage</t>
@@ -166,7 +166,7 @@
     <t>de/de/kinder-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:06.100Z</t>
+    <t>2026-10-21T22:31:25.780Z</t>
   </si>
   <si>
     <t>Mit Kindern und Babys an Bord | Lufthansa</t>
@@ -181,7 +181,7 @@
     <t>de/de/kindermenues-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:08.100Z</t>
+    <t>2026-10-21T22:31:30.745Z</t>
   </si>
   <si>
     <t>Kindermenüs | Lufthansa</t>
@@ -196,7 +196,7 @@
     <t>de/de/lufthansa-first-class-entertainment</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:10.363Z</t>
+    <t>2026-10-21T22:34:02.541Z</t>
   </si>
   <si>
     <t>Entertainment Welt | Lufthansa</t>
@@ -211,7 +211,7 @@
     <t>de/de/lufthansa-first-class-komfort</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:07.683Z</t>
+    <t>2026-10-21T22:32:46.333Z</t>
   </si>
   <si>
     <t>Komfort an Bord der First Class | Lufthansa</t>
@@ -226,7 +226,7 @@
     <t>de/de/menues-auf-langstreckenfluegen</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:13.801Z</t>
+    <t>2026-10-21T22:34:20.948Z</t>
   </si>
   <si>
     <t>Menüs auf Langstreckenflügen | Lufthansa</t>
@@ -241,7 +241,7 @@
     <t>de/de/menues-reiseklassen</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:16.384Z</t>
+    <t>2026-10-21T22:34:25.475Z</t>
   </si>
   <si>
     <t>Menüs in unseren Reiseklassen | Lufthansa</t>
@@ -271,7 +271,7 @@
     <t>de/de/onboard-delights-faq</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:10.658Z</t>
+    <t>2026-10-21T22:32:11.489Z</t>
   </si>
   <si>
     <t>faq | Lufthansa</t>
@@ -289,7 +289,7 @@
     <t>de/de/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:18.569Z</t>
+    <t>2026-10-21T22:34:32.444Z</t>
   </si>
   <si>
     <t>Onboard Delights | Lufthansa</t>
@@ -310,7 +310,7 @@
     <t>hub</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:17.458Z</t>
+    <t>2026-10-21T22:29:36.688Z</t>
   </si>
   <si>
     <t>Services an Bord | Lufthansa</t>
@@ -328,7 +328,7 @@
     <t>de/de/speisen-und-getraenke</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:14.861Z</t>
+    <t>2026-10-21T22:29:10.255Z</t>
   </si>
   <si>
     <t>Menüs an Bord | Lufthansa</t>
@@ -343,7 +343,7 @@
     <t>de/de/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:12.411Z</t>
+    <t>2026-10-21T22:34:47.115Z</t>
   </si>
   <si>
     <t>Unterhaltung an Bord | Lufthansa</t>
@@ -364,7 +364,7 @@
     <t>campaign</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:07.829Z</t>
+    <t>2026-10-21T22:34:52.969Z</t>
   </si>
   <si>
     <t>100 Years Lufthansa | Lufthansa</t>
@@ -385,7 +385,7 @@
     <t>fleet</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:12.414Z</t>
+    <t>2026-10-21T22:35:08.686Z</t>
   </si>
   <si>
     <t>Airbus A350-900 | Lufthansa</t>
@@ -403,7 +403,7 @@
     <t>de/en/accessible-travel</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:22.603Z</t>
+    <t>2026-10-21T22:29:47.559Z</t>
   </si>
   <si>
     <t>Accessible travel | Lufthansa</t>
@@ -418,7 +418,7 @@
     <t>de/en/add-sports-baggage</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:24.619Z</t>
+    <t>2026-10-21T22:29:49.905Z</t>
   </si>
   <si>
     <t>Add sports baggage | Lufthansa</t>
@@ -433,7 +433,7 @@
     <t>de/en/additional-services</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:31.376Z</t>
+    <t>2026-10-21T22:28:54.578Z</t>
   </si>
   <si>
     <t>Extra services | Lufthansa</t>
@@ -448,7 +448,7 @@
     <t>de/en/addresses-worldwide</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:26.855Z</t>
+    <t>2026-10-21T22:29:51.608Z</t>
   </si>
   <si>
     <t>Addresses worldwide | Lufthansa</t>
@@ -463,7 +463,7 @@
     <t>de/en/admission-rules</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:29.362Z</t>
+    <t>2026-10-21T22:29:53.742Z</t>
   </si>
   <si>
     <t>Access to our lounges | Lufthansa</t>
@@ -478,7 +478,7 @@
     <t>de/en/advance-seat-reservation</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:31.443Z</t>
+    <t>2026-10-21T22:29:57.170Z</t>
   </si>
   <si>
     <t>Advance seat reservation | Lufthansa</t>
@@ -496,7 +496,7 @@
     <t>de/en/advice-for-travellers-with-special-needs-to-and-from-the-usa</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:34.110Z</t>
+    <t>2026-10-21T22:29:59.570Z</t>
   </si>
   <si>
     <t>Information about accessible travel to the USA | Lufthansa</t>
@@ -511,7 +511,7 @@
     <t>de/en/affiliatemarketing</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:35.831Z</t>
+    <t>2026-10-21T22:30:02.705Z</t>
   </si>
   <si>
     <t>Affiliate marketing | Lufthansa</t>
@@ -526,7 +526,7 @@
     <t>de/en/airport-information</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:33.884Z</t>
+    <t>2026-10-21T22:28:57.157Z</t>
   </si>
   <si>
     <t>Airport information | Lufthansa</t>
@@ -541,7 +541,7 @@
     <t>de/en/all-check-in</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:37.770Z</t>
+    <t>2026-10-21T22:30:05.727Z</t>
   </si>
   <si>
     <t>All check-in options | Lufthansa</t>
@@ -556,7 +556,7 @@
     <t>de/en/arrival-services</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:39.836Z</t>
+    <t>2026-10-21T22:30:08.819Z</t>
   </si>
   <si>
     <t>Arrival services | Lufthansa</t>
@@ -571,7 +571,7 @@
     <t>de/en/assistenzhunde</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:42.444Z</t>
+    <t>2026-10-21T22:30:11.883Z</t>
   </si>
   <si>
     <t>Assistance dogs | Lufthansa</t>
@@ -586,7 +586,7 @@
     <t>de/en/automatic-check-in</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:44.459Z</t>
+    <t>2026-10-21T22:30:14.648Z</t>
   </si>
   <si>
     <t>Automated check-in | Lufthansa</t>
@@ -604,7 +604,7 @@
     <t>de/en/baggage-irregularities</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:46.494Z</t>
+    <t>2026-10-21T22:30:16.983Z</t>
   </si>
   <si>
     <t>Problems with baggage | Lufthansa</t>
@@ -622,7 +622,7 @@
     <t>de/en/baggage</t>
   </si>
   <si>
-    <t>2026-10-21T16:54:59.566Z</t>
+    <t>2026-10-21T22:28:51.748Z</t>
   </si>
   <si>
     <t>Baggage | Lufthansa</t>
@@ -637,7 +637,7 @@
     <t>de/en/bid-upgrade</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:48.493Z</t>
+    <t>2026-10-21T22:30:19.821Z</t>
   </si>
   <si>
     <t>Submit an offer for your upgrade | Lufthansa</t>
@@ -652,7 +652,7 @@
     <t>de/en/boarding</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:47.048Z</t>
+    <t>2026-10-21T22:30:22.222Z</t>
   </si>
   <si>
     <t>Boarding | Lufthansa</t>
@@ -667,7 +667,7 @@
     <t>de/en/business-class-on-short-and-medium-haul</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:06.858Z</t>
+    <t>2026-10-21T22:31:03.113Z</t>
   </si>
   <si>
     <t>Business Class on short and medium-haul routes | Lufthansa</t>
@@ -682,7 +682,7 @@
     <t>de/en/business-class</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:53.691Z</t>
+    <t>2026-10-21T22:31:00.658Z</t>
   </si>
   <si>
     <t>Business Class | Lufthansa</t>
@@ -697,7 +697,7 @@
     <t>de/en/business-services</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:09.743Z</t>
+    <t>2026-10-21T22:31:05.036Z</t>
   </si>
   <si>
     <t>Business Services | Lufthansa</t>
@@ -712,7 +712,7 @@
     <t>de/en/cancellations-and-refunds</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:11.729Z</t>
+    <t>2026-10-21T22:31:08.458Z</t>
   </si>
   <si>
     <t>Cancellation and refund | Lufthansa</t>
@@ -730,7 +730,7 @@
     <t>de/en/carry-on-baggage</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:14.342Z</t>
+    <t>2026-10-21T22:31:10.950Z</t>
   </si>
   <si>
     <t>Carry-on baggage | Lufthansa</t>
@@ -745,7 +745,7 @@
     <t>de/en/cash-and-miles</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:16.728Z</t>
+    <t>2026-10-21T22:31:14.017Z</t>
   </si>
   <si>
     <t>Cash &amp; Miles | Lufthansa</t>
@@ -760,7 +760,7 @@
     <t>de/en/check-in-baggage</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:18.964Z</t>
+    <t>2026-10-21T22:31:16.993Z</t>
   </si>
   <si>
     <t>Baggage drop | Lufthansa</t>
@@ -775,7 +775,7 @@
     <t>de/en/check-in-with-the-family</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:21.159Z</t>
+    <t>2026-10-21T22:31:18.810Z</t>
   </si>
   <si>
     <t>Online check-in with the whole family | Lufthansa</t>
@@ -790,7 +790,7 @@
     <t>de/en/child-restraint-systems</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:23.683Z</t>
+    <t>2026-10-21T22:31:20.992Z</t>
   </si>
   <si>
     <t>Safety for small children on board | Lufthansa</t>
@@ -805,7 +805,7 @@
     <t>de/en/children-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:50.216Z</t>
+    <t>2026-10-21T22:31:23.009Z</t>
   </si>
   <si>
     <t>On board with children and babies | Lufthansa</t>
@@ -820,7 +820,7 @@
     <t>de/en/childrens-menus-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:52.343Z</t>
+    <t>2026-10-21T22:31:28.164Z</t>
   </si>
   <si>
     <t>Children’s menus | Lufthansa</t>
@@ -835,7 +835,7 @@
     <t>de/en/dangerous-dogs</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:26.211Z</t>
+    <t>2026-10-21T22:31:34.059Z</t>
   </si>
   <si>
     <t>Fighting dog breeds and snub-nosed animals | Lufthansa</t>
@@ -850,7 +850,7 @@
     <t>de/en/digital-baggage-services</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:28.253Z</t>
+    <t>2026-10-21T22:31:36.282Z</t>
   </si>
   <si>
     <t>Digital baggage services | Lufthansa</t>
@@ -865,7 +865,7 @@
     <t>de/en/digital-self-services</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:36.360Z</t>
+    <t>2026-10-21T22:29:00.047Z</t>
   </si>
   <si>
     <t>Digital services | Lufthansa</t>
@@ -880,7 +880,7 @@
     <t>de/en/digital-travel-companion</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:30.083Z</t>
+    <t>2026-10-21T22:31:39.166Z</t>
   </si>
   <si>
     <t>Lufthansa app | Lufthansa</t>
@@ -895,7 +895,7 @@
     <t>de/en/doctor-on-board-news</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:46.896Z</t>
+    <t>2026-10-21T22:32:03.500Z</t>
   </si>
   <si>
     <t>Doctor on Board—good to know | Lufthansa</t>
@@ -910,7 +910,7 @@
     <t>de/en/doctor-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:44.039Z</t>
+    <t>2026-10-21T22:31:58.785Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/doctor-on-board</t>
@@ -922,7 +922,7 @@
     <t>de/en/economy-class</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:47.420Z</t>
+    <t>2026-10-21T22:32:21.285Z</t>
   </si>
   <si>
     <t>Economy Class | Lufthansa</t>
@@ -937,7 +937,7 @@
     <t>de/en/electronic-bag-tags</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:49.689Z</t>
+    <t>2026-10-21T22:32:23.940Z</t>
   </si>
   <si>
     <t>Electronic bag tags | Lufthansa</t>
@@ -952,7 +952,7 @@
     <t>de/en/entryprocesses</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:51.447Z</t>
+    <t>2026-10-21T22:32:26.708Z</t>
   </si>
   <si>
     <t>Entry regulations | Lufthansa</t>
@@ -967,7 +967,7 @@
     <t>de/en/europa-tarife-economy-class</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:53.242Z</t>
+    <t>2026-10-21T22:32:28.714Z</t>
   </si>
   <si>
     <t>Our Europe fares | Lufthansa</t>
@@ -982,7 +982,7 @@
     <t>de/en/europcar</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:55.653Z</t>
+    <t>2026-10-21T22:32:31.567Z</t>
   </si>
   <si>
     <t>Europcar | Lufthansa</t>
@@ -997,7 +997,7 @@
     <t>de/en/exclusive-charter</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:57.587Z</t>
+    <t>2026-10-21T22:32:33.293Z</t>
   </si>
   <si>
     <t>Lufthansa Charter | Lufthansa</t>
@@ -1012,7 +1012,7 @@
     <t>de/en/faq-ejournals</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:59.675Z</t>
+    <t>2026-10-21T22:32:35.654Z</t>
   </si>
   <si>
     <t>FAQs about eJournals | Lufthansa</t>
@@ -1033,7 +1033,7 @@
     <t>form</t>
   </si>
   <si>
-    <t>2026-10-21T17:01:26.038Z</t>
+    <t>2026-10-21T22:35:24.617Z</t>
   </si>
   <si>
     <t>Feedback and other contact forms | Lufthansa</t>
@@ -1048,7 +1048,7 @@
     <t>de/en/fia-valet-service</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:02.056Z</t>
+    <t>2026-10-21T22:32:38.408Z</t>
   </si>
   <si>
     <t>FIA Valet Service | Lufthansa</t>
@@ -1063,7 +1063,7 @@
     <t>de/en/first-class-comfort</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:51.510Z</t>
+    <t>2026-10-21T22:32:43.359Z</t>
   </si>
   <si>
     <t>Comfort on board First Class | Lufthansa</t>
@@ -1081,7 +1081,7 @@
     <t>de/en/first-class-lounges</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:07.253Z</t>
+    <t>2026-10-21T22:32:48.150Z</t>
   </si>
   <si>
     <t>First Class Lounges | Lufthansa</t>
@@ -1096,7 +1096,7 @@
     <t>de/en/first-class-personal-assistant</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:09.619Z</t>
+    <t>2026-10-21T22:32:49.855Z</t>
   </si>
   <si>
     <t>First Class personal assistant service | Lufthansa</t>
@@ -1111,7 +1111,7 @@
     <t>de/en/first-class-terminal</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:11.882Z</t>
+    <t>2026-10-21T22:32:52.460Z</t>
   </si>
   <si>
     <t>First Class Terminal | Lufthansa</t>
@@ -1126,7 +1126,7 @@
     <t>de/en/first-class-valet-parking-service</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:13.849Z</t>
+    <t>2026-10-21T22:32:55.683Z</t>
   </si>
   <si>
     <t>Valet parking service | Lufthansa</t>
@@ -1141,7 +1141,7 @@
     <t>de/en/first-class</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:04.433Z</t>
+    <t>2026-10-21T22:32:40.870Z</t>
   </si>
   <si>
     <t>Lufthansa First Class | Lufthansa</t>
@@ -1156,7 +1156,7 @@
     <t>de/en/fliegen-mit-baby</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:15.560Z</t>
+    <t>2026-10-21T22:32:58.220Z</t>
   </si>
   <si>
     <t>Flying with baby | Lufthansa</t>
@@ -1171,7 +1171,7 @@
     <t>de/en/flight-disruptions</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:17.617Z</t>
+    <t>2026-10-21T22:33:00.710Z</t>
   </si>
   <si>
     <t>Flights delayed and cancelled at short notice | Lufthansa</t>
@@ -1189,7 +1189,7 @@
     <t>de/en/flights</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:40.917Z</t>
+    <t>2026-10-21T22:29:04.966Z</t>
   </si>
   <si>
     <t>Flight offers and destinations worldwide | Lufthansa</t>
@@ -1204,7 +1204,7 @@
     <t>de/en/fly-more-sustainabl</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:20.317Z</t>
+    <t>2026-10-21T22:33:02.743Z</t>
   </si>
   <si>
     <t>Fly more sustainably | Lufthansa</t>
@@ -1219,7 +1219,7 @@
     <t>de/en/flying-with-small-children</t>
   </si>
   <si>
-    <t>2026-10-21T17:01:18.757Z</t>
+    <t>2026-10-21T22:29:44.690Z</t>
   </si>
   <si>
     <t>Flying with small children | Lufthansa</t>
@@ -1234,7 +1234,7 @@
     <t>de/en/flynet</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:46.105Z</t>
+    <t>2026-10-21T22:33:05.112Z</t>
   </si>
   <si>
     <t>FlyNet® on board | Lufthansa</t>
@@ -1249,7 +1249,7 @@
     <t>de/en/fmg-valet-parking-service</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:48.875Z</t>
+    <t>2026-10-21T22:33:07.569Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/fmg-valet-parking-service</t>
@@ -1261,7 +1261,7 @@
     <t>de/en/food-and-beverages</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:43.683Z</t>
+    <t>2026-10-21T22:29:08.014Z</t>
   </si>
   <si>
     <t>Menus on board | Lufthansa</t>
@@ -1288,7 +1288,7 @@
     <t>de/en/free2move</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:51.672Z</t>
+    <t>2026-10-21T22:33:09.325Z</t>
   </si>
   <si>
     <t>Free2move carsharing | Lufthansa</t>
@@ -1303,7 +1303,7 @@
     <t>de/en/freigepaeck-regeln</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:53.913Z</t>
+    <t>2026-10-21T22:33:12.161Z</t>
   </si>
   <si>
     <t>Free baggage rules at Lufthansa | Lufthansa</t>
@@ -1318,7 +1318,7 @@
     <t>de/en/gefaehrliche-gegenstaende</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:57.010Z</t>
+    <t>2026-10-21T22:33:14.892Z</t>
   </si>
   <si>
     <t>Dangerous goods | Lufthansa</t>
@@ -1333,7 +1333,7 @@
     <t>de/en/green-fare</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:59.988Z</t>
+    <t>2026-10-21T22:33:16.852Z</t>
   </si>
   <si>
     <t>Green Fares: More sustainable air travel | Lufthansa</t>
@@ -1348,7 +1348,7 @@
     <t>de/en/group-travel-and-charter</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:04.849Z</t>
+    <t>2026-10-21T22:33:21.847Z</t>
   </si>
   <si>
     <t>Group travel and Lufthansa Charter | Lufthansa</t>
@@ -1363,7 +1363,7 @@
     <t>de/en/group-travel</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:02.306Z</t>
+    <t>2026-10-21T22:33:19.066Z</t>
   </si>
   <si>
     <t>Group travel | Lufthansa</t>
@@ -1378,7 +1378,7 @@
     <t>de/en/hertz</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:07.686Z</t>
+    <t>2026-10-21T22:33:24.343Z</t>
   </si>
   <si>
     <t>Hertz | Lufthansa</t>
@@ -1393,7 +1393,7 @@
     <t>de/en/homepage</t>
   </si>
   <si>
-    <t>2026-10-21T22:28:36.795Z</t>
+    <t>2026-10-22T00:04:28.208Z</t>
   </si>
   <si>
     <t>Book your flight now - travel with Lufthansa to over 200 destinations | Lufthansa</t>
@@ -1408,7 +1408,7 @@
     <t>de/en/hotel-offers</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:10.223Z</t>
+    <t>2026-10-21T22:33:26.676Z</t>
   </si>
   <si>
     <t>Hotel offers | Lufthansa</t>
@@ -1429,7 +1429,7 @@
     <t>legal</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:21.743Z</t>
+    <t>2026-10-21T22:35:19.333Z</t>
   </si>
   <si>
     <t>Legal notice | Lufthansa</t>
@@ -1444,7 +1444,7 @@
     <t>de/en/lh-rentalcar</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:12.065Z</t>
+    <t>2026-10-21T22:33:29.136Z</t>
   </si>
   <si>
     <t>Car rental partners | Lufthansa</t>
@@ -1459,7 +1459,7 @@
     <t>de/en/lounge-companions</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:14.309Z</t>
+    <t>2026-10-21T22:33:31.893Z</t>
   </si>
   <si>
     <t>Take your companions into the lounge with you | Lufthansa</t>
@@ -1474,7 +1474,7 @@
     <t>de/en/lounges</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:46.343Z</t>
+    <t>2026-10-21T22:29:12.311Z</t>
   </si>
   <si>
     <t>Lounges | Lufthansa</t>
@@ -1489,7 +1489,7 @@
     <t>de/en/lufthansa-am-flughafen-frankfurt</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:17.122Z</t>
+    <t>2026-10-21T22:33:33.693Z</t>
   </si>
   <si>
     <t>Lufthansa at Frankfurt Airport | Lufthansa</t>
@@ -1504,7 +1504,7 @@
     <t>de/en/lufthansa-at-berlin-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:20.140Z</t>
+    <t>2026-10-21T22:33:36.028Z</t>
   </si>
   <si>
     <t>Lufthansa at Berlin Brandenburg Airport | Lufthansa</t>
@@ -1519,7 +1519,7 @@
     <t>de/en/lufthansa-at-duesseldorf-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:21.964Z</t>
+    <t>2026-10-21T22:33:38.951Z</t>
   </si>
   <si>
     <t>Lufthansa at Dusseldorf Airport | Lufthansa</t>
@@ -1534,7 +1534,7 @@
     <t>de/en/lufthansa-at-vienna-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:24.577Z</t>
+    <t>2026-10-21T22:33:41.420Z</t>
   </si>
   <si>
     <t>Lufthansa at Vienna Airport | Lufthansa</t>
@@ -1549,7 +1549,7 @@
     <t>de/en/lufthansa-at-zuerich-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:26.731Z</t>
+    <t>2026-10-21T22:33:43.859Z</t>
   </si>
   <si>
     <t>Lufthansa at Zurich Airport | Lufthansa</t>
@@ -1564,7 +1564,7 @@
     <t>de/en/lufthansa-aviation-group</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:29.559Z</t>
+    <t>2026-10-21T22:33:45.803Z</t>
   </si>
   <si>
     <t>Lufthansa Aviation Group | Lufthansa</t>
@@ -1579,7 +1579,7 @@
     <t>de/en/lufthansa-business-class-on-long-haul-routes</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:15.868Z</t>
+    <t>2026-10-21T22:33:48.569Z</t>
   </si>
   <si>
     <t>Business Class on long-haul routes | Lufthansa</t>
@@ -1594,7 +1594,7 @@
     <t>de/en/lufthansa-corporate-customers</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:18.993Z</t>
+    <t>2026-10-21T22:33:50.458Z</t>
   </si>
   <si>
     <t>Lufthansa for corporate customers | Lufthansa</t>
@@ -1609,7 +1609,7 @@
     <t>de/en/lufthansa-express-bus</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:24.413Z</t>
+    <t>2026-10-21T22:33:54.761Z</t>
   </si>
   <si>
     <t>Lufthansa Express Bus | Lufthansa</t>
@@ -1624,7 +1624,7 @@
     <t>de/en/lufthansa-express-rail</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:26.813Z</t>
+    <t>2026-10-21T22:33:56.987Z</t>
   </si>
   <si>
     <t>Lufthansa Express Rail | Lufthansa</t>
@@ -1639,7 +1639,7 @@
     <t>de/en/lufthansa-express</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:22.240Z</t>
+    <t>2026-10-21T22:33:52.450Z</t>
   </si>
   <si>
     <t>Airport arrival and departure – travel seamlessly | Lufthansa</t>
@@ -1654,7 +1654,7 @@
     <t>de/en/lufthansa-first-class-entertainment</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:53.390Z</t>
+    <t>2026-10-21T22:34:00.424Z</t>
   </si>
   <si>
     <t>Entertainment world | Lufthansa</t>
@@ -1669,7 +1669,7 @@
     <t>de/en/lufthansa-group-star-alliance-and-partner-airlines</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:29.393Z</t>
+    <t>2026-10-21T22:34:05.613Z</t>
   </si>
   <si>
     <t>Lufthansa Group, Star Alliance and partner airlines | Lufthansa</t>
@@ -1684,7 +1684,7 @@
     <t>de/en/lufthansa-guide-service</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:31.391Z</t>
+    <t>2026-10-21T22:34:07.304Z</t>
   </si>
   <si>
     <t>Lufthansa Guide Service Munich | Lufthansa</t>
@@ -1699,7 +1699,7 @@
     <t>de/en/lufthansa-terminal-muenchen</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:34.041Z</t>
+    <t>2026-10-21T22:34:10.267Z</t>
   </si>
   <si>
     <t>Lufthansa at Munich Airport | Lufthansa</t>
@@ -1714,7 +1714,7 @@
     <t>de/en/lufthansa-travel-classes</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:49.011Z</t>
+    <t>2026-10-21T22:29:15.410Z</t>
   </si>
   <si>
     <t>Our travel classes | Lufthansa</t>
@@ -1729,7 +1729,7 @@
     <t>de/en/medikamenten-transport</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:35.792Z</t>
+    <t>2026-10-21T22:34:13.158Z</t>
   </si>
   <si>
     <t>Always at the right temperature | Lufthansa</t>
@@ -1744,7 +1744,7 @@
     <t>de/en/meetings-and-events-delegates</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:38.070Z</t>
+    <t>2026-10-21T22:34:15.050Z</t>
   </si>
   <si>
     <t>Meetings &amp; Events: Information for organisers | Lufthansa</t>
@@ -1759,7 +1759,7 @@
     <t>de/en/meetings-and-events-organisers</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:39.756Z</t>
+    <t>2026-10-21T22:34:16.965Z</t>
   </si>
   <si>
     <t>Meeting &amp; Events: Information for organisers | Lufthansa</t>
@@ -1774,7 +1774,7 @@
     <t>de/en/meetings-and-events</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:51.766Z</t>
+    <t>2026-10-21T22:29:17.390Z</t>
   </si>
   <si>
     <t>Lufthansa Group Meetings &amp; Events | Lufthansa</t>
@@ -1789,7 +1789,7 @@
     <t>de/en/menus-on-long-haul-flights</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:56.509Z</t>
+    <t>2026-10-21T22:34:18.943Z</t>
   </si>
   <si>
     <t>Menus on long-haul flights | Lufthansa</t>
@@ -1804,7 +1804,7 @@
     <t>de/en/menus-travel-classes</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:58.485Z</t>
+    <t>2026-10-21T22:34:23.793Z</t>
   </si>
   <si>
     <t>Menus in our travel classes | Lufthansa</t>
@@ -1819,7 +1819,7 @@
     <t>de/en/miles-and-more</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:53.850Z</t>
+    <t>2026-10-21T22:29:19.875Z</t>
   </si>
   <si>
     <t>Miles &amp; More – Our frequent flyer programme | Lufthansa</t>
@@ -1834,7 +1834,7 @@
     <t>de/en/mobility-partner-program-healthcare</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:41.730Z</t>
+    <t>2026-10-21T22:34:27.573Z</t>
   </si>
   <si>
     <t>Lufthansa Global Healthcare and Medical Services | Lufthansa</t>
@@ -1861,7 +1861,7 @@
     <t>de/en/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:00.742Z</t>
+    <t>2026-10-21T22:34:30.374Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/onboard-delights</t>
@@ -1873,7 +1873,7 @@
     <t>de/en/online-check-in-info</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:44.910Z</t>
+    <t>2026-10-21T22:34:34.662Z</t>
   </si>
   <si>
     <t>Online check-in information | Lufthansa</t>
@@ -1894,7 +1894,7 @@
     <t>app-entry</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:30.108Z</t>
+    <t>2026-10-21T22:35:29.211Z</t>
   </si>
   <si>
     <t>Online check-in | Lufthansa</t>
@@ -1909,7 +1909,7 @@
     <t>de/en/overview-flights</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:55.609Z</t>
+    <t>2026-10-21T22:29:22.394Z</t>
   </si>
   <si>
     <t>Flights – your journey starts here | Lufthansa</t>
@@ -1927,7 +1927,7 @@
     <t>de/en/overview-manage</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:57.674Z</t>
+    <t>2026-10-21T22:29:24.956Z</t>
   </si>
   <si>
     <t>Manage your bookings | Lufthansa</t>
@@ -1942,7 +1942,7 @@
     <t>de/en/overview-special-request</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:59.788Z</t>
+    <t>2026-10-21T22:29:26.725Z</t>
   </si>
   <si>
     <t>Special requests | Lufthansa</t>
@@ -1957,7 +1957,7 @@
     <t>de/en/overview-travel-information</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:02.269Z</t>
+    <t>2026-10-21T22:29:29.135Z</t>
   </si>
   <si>
     <t>Travel information – what you need to know | Lufthansa</t>
@@ -1972,7 +1972,7 @@
     <t>de/en/partner</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:47.324Z</t>
+    <t>2026-10-21T22:34:37.659Z</t>
   </si>
   <si>
     <t>Partners | Lufthansa</t>
@@ -1987,7 +1987,7 @@
     <t>de/en/passenger-receipt-90</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:50.672Z</t>
+    <t>2026-10-21T22:34:39.755Z</t>
   </si>
   <si>
     <t>Passenger receipt | Lufthansa</t>
@@ -2002,7 +2002,7 @@
     <t>de/en/passengers-using-wheelchairs</t>
   </si>
   <si>
-    <t>2026-10-21T22:27:53.194Z</t>
+    <t>2026-10-21T22:34:42.001Z</t>
   </si>
   <si>
     <t>Passengers requiring wheelchairs | Lufthansa</t>
@@ -2011,13 +2011,58 @@
     <t>https://www.lufthansa.com/de/en/passengers-using-wheelchairs</t>
   </si>
   <si>
+    <t>de/en/passengers-with-sensory-impairment.report.json</t>
+  </si>
+  <si>
+    <t>de/en/passengers-with-sensory-impairment</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:02:44.087Z</t>
+  </si>
+  <si>
+    <t>Passengers with sensory impairments | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/passengers-with-sensory-impairment</t>
+  </si>
+  <si>
+    <t>de/en/payment-options-at-the-airport.report.json</t>
+  </si>
+  <si>
+    <t>de/en/payment-options-at-the-airport</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:02:46.372Z</t>
+  </si>
+  <si>
+    <t>Payment options at the airport | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/payment-options-at-the-airport</t>
+  </si>
+  <si>
+    <t>de/en/premium-economy-class.report.json</t>
+  </si>
+  <si>
+    <t>de/en/premium-economy-class</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:02:49.212Z</t>
+  </si>
+  <si>
+    <t>Premium Economy Class | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/premium-economy-class</t>
+  </si>
+  <si>
     <t>de/en/services-at-the-airport.report.json</t>
   </si>
   <si>
     <t>de/en/services-at-the-airport</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:04.410Z</t>
+    <t>2026-10-21T22:29:32.371Z</t>
   </si>
   <si>
     <t>Services at the airport | Lufthansa</t>
@@ -2032,7 +2077,7 @@
     <t>de/en/services-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:06.364Z</t>
+    <t>2026-10-21T22:29:34.558Z</t>
   </si>
   <si>
     <t>Services on board | Lufthansa</t>
@@ -2047,7 +2092,7 @@
     <t>de/en/special-needs</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:09.544Z</t>
+    <t>2026-10-21T22:29:39.318Z</t>
   </si>
   <si>
     <t>Register your assistance requirements online | Lufthansa</t>
@@ -2068,7 +2113,7 @@
     <t>flight-status</t>
   </si>
   <si>
-    <t>2026-10-21T17:01:33.445Z</t>
+    <t>2026-10-21T22:35:34.539Z</t>
   </si>
   <si>
     <t>Timetable &amp; flight status | Lufthansa</t>
@@ -2083,7 +2128,7 @@
     <t>de/en/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:55.435Z</t>
+    <t>2026-10-21T22:34:44.190Z</t>
   </si>
   <si>
     <t>Entertainment on board | Lufthansa</t>
@@ -2110,7 +2155,7 @@
     <t>gb/en/homepage</t>
   </si>
   <si>
-    <t>2026-10-21T22:28:46.096Z</t>
+    <t>2026-10-22T00:04:38.121Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/homepage</t>
@@ -2140,7 +2185,7 @@
     <t>aircore-destination-overview</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:43.571Z</t>
+    <t>2026-10-21T22:35:43.227Z</t>
   </si>
   <si>
     <t>Book flights to destinations all over the world | Lufthansa</t>
@@ -2173,7 +2218,7 @@
     <t>de/de/discover-lufthansa/new-onboard-experience</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:27.478Z</t>
+    <t>2026-10-21T22:35:03.116Z</t>
   </si>
   <si>
     <t>New Onboard Experience | Lufthansa</t>
@@ -2188,7 +2233,7 @@
     <t>de/de/during-your-trip/lhg-wifi</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:04.970Z</t>
+    <t>2026-10-21T22:32:18.873Z</t>
   </si>
   <si>
     <t>Lufthansa Group Wi-Fi | Lufthansa</t>
@@ -2215,7 +2260,7 @@
     <t>de/en/book-and-manage/pax-receipt</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:40.390Z</t>
+    <t>2026-10-21T22:30:46.923Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/book-and-manage/pax-receipt</t>
@@ -2227,7 +2272,7 @@
     <t>de/en/book-and-manage/rebook</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:46.117Z</t>
+    <t>2026-10-21T22:30:52.704Z</t>
   </si>
   <si>
     <t>Flight Rebooking | Lufthansa</t>
@@ -2242,7 +2287,7 @@
     <t>de/en/discover-lufthansa/flightreservation-priceguarantee</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:42.460Z</t>
+    <t>2026-10-21T22:31:51.511Z</t>
   </si>
   <si>
     <t>Reservation with price guarantee | Lufthansa</t>
@@ -2257,7 +2302,7 @@
     <t>de/en/discover-lufthansa/miles-and-more-credit-card</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:46.716Z</t>
+    <t>2026-10-21T22:31:56.206Z</t>
   </si>
   <si>
     <t>Miles &amp; More Credit Card | Lufthansa</t>
@@ -2272,7 +2317,7 @@
     <t>de/en/discover-lufthansa/new-onboard-experience</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:19.974Z</t>
+    <t>2026-10-21T22:34:59.894Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/discover-lufthansa/new-onboard-experience</t>
@@ -2284,7 +2329,7 @@
     <t>de/en/during-your-trip/internet-overview</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:44.425Z</t>
+    <t>2026-10-21T22:32:14.040Z</t>
   </si>
   <si>
     <t>Internet | Lufthansa</t>
@@ -2299,7 +2344,7 @@
     <t>de/en/during-your-trip/lhg-wifi</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:48.988Z</t>
+    <t>2026-10-21T22:32:16.809Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/during-your-trip/lhg-wifi</t>
@@ -2317,6 +2362,21 @@
     <t>https://www.lufthansa.com/de/en/homepage#payment-social</t>
   </si>
   <si>
+    <t>de/en/prepare-for-your-trip/current-travel-information.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/current-travel-information</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:04.692Z</t>
+  </si>
+  <si>
+    <t>Current information | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/current-travel-information</t>
+  </si>
+  <si>
     <t>gb/en/fragments/payment-social.report.json</t>
   </si>
   <si>
@@ -2359,7 +2419,7 @@
     <t>de/de/100-years/history/menu-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:24.361Z</t>
+    <t>2026-10-21T22:34:57.145Z</t>
   </si>
   <si>
     <t>Menüs an Board | Lufthansa</t>
@@ -2374,7 +2434,7 @@
     <t>de/en/100-years/history/menu-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:17.824Z</t>
+    <t>2026-10-21T22:34:54.910Z</t>
   </si>
   <si>
     <t>Menus on Board | Lufthansa</t>
@@ -2395,7 +2455,7 @@
     <t>insights</t>
   </si>
   <si>
-    <t>2026-10-21T16:55:17.564Z</t>
+    <t>2026-10-21T22:35:13.632Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/articles/explore-the-world/eat-see-do-berlin</t>
@@ -2407,7 +2467,7 @@
     <t>de/en/book-and-manage/additional-services/get-your-guide</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:49.789Z</t>
+    <t>2026-10-21T22:30:23.858Z</t>
   </si>
   <si>
     <t>Unforgettable travel experiences—GetYourGuide | Lufthansa</t>
@@ -2422,7 +2482,7 @@
     <t>de/en/book-and-manage/additional-services/travel-insurances</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:51.782Z</t>
+    <t>2026-10-21T22:30:26.033Z</t>
   </si>
   <si>
     <t>Travel Care | Lufthansa</t>
@@ -2437,7 +2497,7 @@
     <t>de/en/book-and-manage/digital-self-services/airline-apps</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:54.185Z</t>
+    <t>2026-10-21T22:30:27.759Z</t>
   </si>
   <si>
     <t>Simply travel smarter | Lufthansa</t>
@@ -2452,7 +2512,7 @@
     <t>de/en/book-and-manage/flights/air-baltic</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:56.300Z</t>
+    <t>2026-10-21T22:30:30.294Z</t>
   </si>
   <si>
     <t>Your Lufthansa flight with airBaltic | Lufthansa</t>
@@ -2467,7 +2527,7 @@
     <t>de/en/book-and-manage/flights/ana</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:58.144Z</t>
+    <t>2026-10-21T22:30:32.649Z</t>
   </si>
   <si>
     <t>ANA | Lufthansa</t>
@@ -2485,7 +2545,7 @@
     <t>de/en/book-and-manage/flights/giftvoucher</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:31.410Z</t>
+    <t>2026-10-21T22:30:37.799Z</t>
   </si>
   <si>
     <t>Buy a Lufthansa Gift Card &amp; give a flight as a gift | Lufthansa</t>
@@ -2500,7 +2560,7 @@
     <t>de/en/book-and-manage/flights/helvetic</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:33.522Z</t>
+    <t>2026-10-21T22:30:40.563Z</t>
   </si>
   <si>
     <t>Helvetic | Lufthansa</t>
@@ -2515,7 +2575,7 @@
     <t>de/en/book-and-manage/flights/lufthansa-voucher</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:35.591Z</t>
+    <t>2026-10-21T22:30:43.081Z</t>
   </si>
   <si>
     <t>Terms of use for the purchase of Gift Vouchers | Lufthansa</t>
@@ -2530,7 +2590,7 @@
     <t>de/en/book-and-manage/flights/wetlease-hub</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:37.711Z</t>
+    <t>2026-10-21T22:30:44.869Z</t>
   </si>
   <si>
     <t>Wet lease flights | Lufthansa</t>
@@ -2545,7 +2605,7 @@
     <t>de/en/book-and-manage/pax-receipt/invoices-different-countries</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:43.197Z</t>
+    <t>2026-10-21T22:30:49.989Z</t>
   </si>
   <si>
     <t>Invoices for different countries | Lufthansa</t>
@@ -2560,7 +2620,7 @@
     <t>de/en/book-and-manage/rebook/involuntary-rebooking</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:49.236Z</t>
+    <t>2026-10-21T22:30:55.679Z</t>
   </si>
   <si>
     <t>Flight cancellation | Lufthansa</t>
@@ -2575,7 +2635,7 @@
     <t>de/en/book-and-manage/rebook/voluntary-rebooking</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:51.326Z</t>
+    <t>2026-10-21T22:30:57.574Z</t>
   </si>
   <si>
     <t>Change flight | Lufthansa</t>
@@ -2590,7 +2650,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/climate-protection-projects</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:33.023Z</t>
+    <t>2026-10-21T22:31:42.262Z</t>
   </si>
   <si>
     <t>Climate protection projects | Lufthansa</t>
@@ -2605,7 +2665,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/environmental-cost-surcharge</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:35.658Z</t>
+    <t>2026-10-21T22:31:44.526Z</t>
   </si>
   <si>
     <t>Environmental Cost Surcharge | Lufthansa</t>
@@ -2620,7 +2680,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/faq-saf</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:37.765Z</t>
+    <t>2026-10-21T22:31:47.219Z</t>
   </si>
   <si>
     <t>FAQs Sustainable Aviation Fuel | Lufthansa</t>
@@ -2635,7 +2695,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/saf</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:40.111Z</t>
+    <t>2026-10-21T22:31:49.735Z</t>
   </si>
   <si>
     <t>Why support the use of Sustainable Aviation Fuel? | Lufthansa</t>
@@ -2650,7 +2710,7 @@
     <t>de/en/discover-lufthansa/lufthansa-group-airlines/ita-airways</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:44.302Z</t>
+    <t>2026-10-21T22:31:53.994Z</t>
   </si>
   <si>
     <t>ITA Airways | Lufthansa</t>
@@ -2659,6 +2719,96 @@
     <t>https://www.lufthansa.com/de/en/discover-lufthansa/lufthansa-group-airlines/ita-airways</t>
   </si>
   <si>
+    <t>de/en/prepare-for-your-trip/baggage/electronic-devices-and-batteries.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/baggage/electronic-devices-and-batteries</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:01.487Z</t>
+  </si>
+  <si>
+    <t>Electronic devices and batteries | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/baggage/electronic-devices-and-batteries</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/entry-regulations/immigration-regulations-uk.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/entry-regulations/immigration-regulations-uk</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:09.673Z</t>
+  </si>
+  <si>
+    <t>New entry regulations for the United Kingdom | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/entry-regulations/immigration-regulations-uk</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/getting-to-and-from-the-airport/lufthansa-express-bus-briefing.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/getting-to-and-from-the-airport/lufthansa-express-bus-briefing</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:11.398Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Express Bus – assuring your journey | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/getting-to-and-from-the-airport/lufthansa-express-bus-briefing</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/getting-to-and-from-the-airport/lufthansa-express-rail-briefing.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/getting-to-and-from-the-airport/lufthansa-express-rail-briefing</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:13.929Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Express Rail – assuring your journey | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/getting-to-and-from-the-airport/lufthansa-express-rail-briefing</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/medical-travel-companions.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/medical-travel-companions</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:16.155Z</t>
+  </si>
+  <si>
+    <t>Medical travel companions | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/special-travel-needs/medical-travel-companions</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/travel-classes/economy-basic.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/travel-classes/economy-basic</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:28.522Z</t>
+  </si>
+  <si>
+    <t>Economy Basic | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/travel-classes/economy-basic</t>
+  </si>
+  <si>
     <t>de/en/book-and-manage/flights/ana/faq.report.json</t>
   </si>
   <si>
@@ -2668,7 +2818,7 @@
     <t>de/en/book-and-manage/flights/ana/faq</t>
   </si>
   <si>
-    <t>2026-10-21T20:42:00.121Z</t>
+    <t>2026-10-21T22:30:35.269Z</t>
   </si>
   <si>
     <t>FAQs on travel with Lufthansa and ANA | Lufthansa</t>
@@ -2683,7 +2833,7 @@
     <t>de/en/during-your-trip/food-and-beverages/onboard-delights/faq</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:54.738Z</t>
+    <t>2026-10-21T22:32:08.618Z</t>
   </si>
   <si>
     <t>FAQs | Lufthansa</t>
@@ -2692,6 +2842,126 @@
     <t>https://www.lufthansa.com/de/en/during-your-trip/food-and-beverages/onboard-delights/faq</t>
   </si>
   <si>
+    <t>de/en/prepare-for-your-trip/baggage/baggage-irregularities/delayed-baggage-lhg.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/baggage/baggage-irregularities/delayed-baggage-lhg</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:02:51.834Z</t>
+  </si>
+  <si>
+    <t>Delayed baggage lhg | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/baggage/baggage-irregularities/delayed-baggage-lhg</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/baggage/baggage-irregularities/faq-baggage-delay.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/baggage/baggage-irregularities/faq-baggage-delay</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:02:55.363Z</t>
+  </si>
+  <si>
+    <t>Frequently asked questions about delayed baggage | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/baggage/baggage-irregularities/faq-baggage-delay</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/baggage/baggage-irregularities/faq-damaged-baggage.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/baggage/baggage-irregularities/faq-damaged-baggage</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:02:58.415Z</t>
+  </si>
+  <si>
+    <t>Frequently asked questions about damaged baggage | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/baggage/baggage-irregularities/faq-damaged-baggage</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/entry-regulations/entering-schengen/entry-exit-system.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/entry-regulations/entering-schengen/entry-exit-system</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:07.347Z</t>
+  </si>
+  <si>
+    <t>EES: the European Union’s new Entry/Exit System | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/entry-regulations/entering-schengen/entry-exit-system</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/cognitive-impairment.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/cognitive-impairment</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:18.292Z</t>
+  </si>
+  <si>
+    <t>Cognitive impairments | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/cognitive-impairment</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/hearing-impairment.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/hearing-impairment</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:20.474Z</t>
+  </si>
+  <si>
+    <t>Hearing impairments | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/hearing-impairment</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/travel-companion.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/travel-companion</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:23.312Z</t>
+  </si>
+  <si>
+    <t>Travelling with a companion | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/travel-companion</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/visual-impairment.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/visual-impairment</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:03:26.446Z</t>
+  </si>
+  <si>
+    <t>Visual impairments | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/special-travel-needs/travel-with-needs/visual-impairment</t>
+  </si>
+  <si>
     <t>lhg/de/en/dest/cy/new-york.report.json</t>
   </si>
   <si>
@@ -2701,7 +2971,7 @@
     <t>lhg/de/en/dest/cy/new-york</t>
   </si>
   <si>
-    <t>2026-10-21T17:07:20.550Z</t>
+    <t>2026-10-21T22:35:49.019Z</t>
   </si>
   <si>
     <t>Flight to New York (NYC) | Lufthansa</t>
@@ -2722,7 +2992,7 @@
     <t>aircore-route</t>
   </si>
   <si>
-    <t>2026-10-21T17:07:24.799Z</t>
+    <t>2026-10-21T22:35:55.034Z</t>
   </si>
   <si>
     <t>Flights from Germany to USA | Lufthansa</t>
@@ -3117,7 +3387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I175"/>
+  <dimension ref="A1:I193"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -6857,7 +7127,7 @@
         <v>13</v>
       </c>
       <c r="F129" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G129" t="s">
         <v>668</v>
@@ -6874,7 +7144,7 @@
         <v>671</v>
       </c>
       <c r="B130" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="C130" t="s">
         <v>10</v>
@@ -6886,7 +7156,7 @@
         <v>13</v>
       </c>
       <c r="F130" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G130" t="s">
         <v>673</v>
@@ -6915,7 +7185,7 @@
         <v>13</v>
       </c>
       <c r="F131" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G131" t="s">
         <v>678</v>
@@ -6932,94 +7202,94 @@
         <v>681</v>
       </c>
       <c r="B132" t="s">
+        <v>36</v>
+      </c>
+      <c r="C132" t="s">
+        <v>10</v>
+      </c>
+      <c r="D132" t="s">
         <v>682</v>
       </c>
-      <c r="C132" t="s">
-        <v>10</v>
-      </c>
-      <c r="D132" t="s">
+      <c r="E132" t="s">
+        <v>13</v>
+      </c>
+      <c r="F132" t="s">
+        <v>98</v>
+      </c>
+      <c r="G132" t="s">
         <v>683</v>
       </c>
-      <c r="E132" t="s">
-        <v>13</v>
-      </c>
-      <c r="F132" t="s">
+      <c r="H132" t="s">
         <v>684</v>
       </c>
-      <c r="G132" t="s">
+      <c r="I132" t="s">
         <v>685</v>
-      </c>
-      <c r="H132" t="s">
-        <v>686</v>
-      </c>
-      <c r="I132" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
+        <v>686</v>
+      </c>
+      <c r="B133" t="s">
+        <v>96</v>
+      </c>
+      <c r="C133" t="s">
+        <v>10</v>
+      </c>
+      <c r="D133" t="s">
+        <v>687</v>
+      </c>
+      <c r="E133" t="s">
+        <v>13</v>
+      </c>
+      <c r="F133" t="s">
+        <v>98</v>
+      </c>
+      <c r="G133" t="s">
         <v>688</v>
       </c>
-      <c r="B133" t="s">
-        <v>36</v>
-      </c>
-      <c r="C133" t="s">
-        <v>10</v>
-      </c>
-      <c r="D133" t="s">
+      <c r="H133" t="s">
         <v>689</v>
       </c>
-      <c r="E133" t="s">
-        <v>13</v>
-      </c>
-      <c r="F133" t="s">
-        <v>31</v>
-      </c>
-      <c r="G133" t="s">
+      <c r="I133" t="s">
         <v>690</v>
-      </c>
-      <c r="H133" t="s">
-        <v>691</v>
-      </c>
-      <c r="I133" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
+        <v>691</v>
+      </c>
+      <c r="B134" t="s">
+        <v>36</v>
+      </c>
+      <c r="C134" t="s">
+        <v>10</v>
+      </c>
+      <c r="D134" t="s">
+        <v>692</v>
+      </c>
+      <c r="E134" t="s">
+        <v>13</v>
+      </c>
+      <c r="F134" t="s">
+        <v>98</v>
+      </c>
+      <c r="G134" t="s">
         <v>693</v>
       </c>
-      <c r="B134" t="s">
-        <v>10</v>
-      </c>
-      <c r="C134" t="s">
-        <v>11</v>
-      </c>
-      <c r="D134" t="s">
+      <c r="H134" t="s">
         <v>694</v>
       </c>
-      <c r="E134" t="s">
-        <v>13</v>
-      </c>
-      <c r="F134" t="s">
-        <v>14</v>
-      </c>
-      <c r="G134" t="s">
+      <c r="I134" t="s">
         <v>695</v>
-      </c>
-      <c r="H134" t="s">
-        <v>10</v>
-      </c>
-      <c r="I134" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
+        <v>696</v>
+      </c>
+      <c r="B135" t="s">
         <v>697</v>
-      </c>
-      <c r="B135" t="s">
-        <v>18</v>
       </c>
       <c r="C135" t="s">
         <v>10</v>
@@ -7031,71 +7301,71 @@
         <v>13</v>
       </c>
       <c r="F135" t="s">
-        <v>20</v>
+        <v>699</v>
       </c>
       <c r="G135" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="H135" t="s">
-        <v>461</v>
+        <v>701</v>
       </c>
       <c r="I135" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="B136" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C136" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D136" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="E136" t="s">
         <v>13</v>
       </c>
       <c r="F136" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G136" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="H136" t="s">
-        <v>10</v>
+        <v>706</v>
       </c>
       <c r="I136" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="B137" t="s">
-        <v>706</v>
+        <v>10</v>
       </c>
       <c r="C137" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D137" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="E137" t="s">
         <v>13</v>
       </c>
       <c r="F137" t="s">
-        <v>708</v>
+        <v>14</v>
       </c>
       <c r="G137" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="H137" t="s">
-        <v>710</v>
+        <v>10</v>
       </c>
       <c r="I137" t="s">
         <v>711</v>
@@ -7106,97 +7376,97 @@
         <v>712</v>
       </c>
       <c r="B138" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C138" t="s">
+        <v>10</v>
+      </c>
+      <c r="D138" t="s">
         <v>713</v>
       </c>
-      <c r="D138" t="s">
+      <c r="E138" t="s">
+        <v>13</v>
+      </c>
+      <c r="F138" t="s">
+        <v>20</v>
+      </c>
+      <c r="G138" t="s">
         <v>714</v>
       </c>
-      <c r="E138" t="s">
-        <v>13</v>
-      </c>
-      <c r="F138" t="s">
-        <v>14</v>
-      </c>
-      <c r="G138" t="s">
+      <c r="H138" t="s">
+        <v>461</v>
+      </c>
+      <c r="I138" t="s">
         <v>715</v>
-      </c>
-      <c r="H138" t="s">
-        <v>10</v>
-      </c>
-      <c r="I138" t="s">
-        <v>716</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
+        <v>716</v>
+      </c>
+      <c r="B139" t="s">
+        <v>10</v>
+      </c>
+      <c r="C139" t="s">
+        <v>14</v>
+      </c>
+      <c r="D139" t="s">
         <v>717</v>
       </c>
-      <c r="B139" t="s">
+      <c r="E139" t="s">
+        <v>13</v>
+      </c>
+      <c r="F139" t="s">
+        <v>14</v>
+      </c>
+      <c r="G139" t="s">
         <v>718</v>
       </c>
-      <c r="C139" t="s">
-        <v>10</v>
-      </c>
-      <c r="D139" t="s">
+      <c r="H139" t="s">
+        <v>10</v>
+      </c>
+      <c r="I139" t="s">
         <v>719</v>
-      </c>
-      <c r="E139" t="s">
-        <v>13</v>
-      </c>
-      <c r="F139" t="s">
-        <v>116</v>
-      </c>
-      <c r="G139" t="s">
-        <v>720</v>
-      </c>
-      <c r="H139" t="s">
-        <v>721</v>
-      </c>
-      <c r="I139" t="s">
-        <v>722</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
+        <v>720</v>
+      </c>
+      <c r="B140" t="s">
+        <v>721</v>
+      </c>
+      <c r="C140" t="s">
+        <v>10</v>
+      </c>
+      <c r="D140" t="s">
+        <v>722</v>
+      </c>
+      <c r="E140" t="s">
+        <v>13</v>
+      </c>
+      <c r="F140" t="s">
         <v>723</v>
       </c>
-      <c r="B140" t="s">
-        <v>84</v>
-      </c>
-      <c r="C140" t="s">
-        <v>10</v>
-      </c>
-      <c r="D140" t="s">
+      <c r="G140" t="s">
         <v>724</v>
       </c>
-      <c r="E140" t="s">
-        <v>13</v>
-      </c>
-      <c r="F140" t="s">
-        <v>31</v>
-      </c>
-      <c r="G140" t="s">
+      <c r="H140" t="s">
         <v>725</v>
       </c>
-      <c r="H140" t="s">
+      <c r="I140" t="s">
         <v>726</v>
-      </c>
-      <c r="I140" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
+        <v>727</v>
+      </c>
+      <c r="B141" t="s">
+        <v>10</v>
+      </c>
+      <c r="C141" t="s">
         <v>728</v>
-      </c>
-      <c r="B141" t="s">
-        <v>10</v>
-      </c>
-      <c r="C141" t="s">
-        <v>713</v>
       </c>
       <c r="D141" t="s">
         <v>729</v>
@@ -7222,42 +7492,42 @@
         <v>732</v>
       </c>
       <c r="B142" t="s">
-        <v>36</v>
+        <v>733</v>
       </c>
       <c r="C142" t="s">
         <v>10</v>
       </c>
       <c r="D142" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="E142" t="s">
         <v>13</v>
       </c>
       <c r="F142" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="G142" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="H142" t="s">
-        <v>659</v>
+        <v>736</v>
       </c>
       <c r="I142" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="B143" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C143" t="s">
         <v>10</v>
       </c>
       <c r="D143" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="E143" t="s">
         <v>13</v>
@@ -7266,56 +7536,56 @@
         <v>31</v>
       </c>
       <c r="G143" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="H143" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="I143" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B144" t="s">
-        <v>84</v>
+        <v>10</v>
       </c>
       <c r="C144" t="s">
-        <v>10</v>
+        <v>728</v>
       </c>
       <c r="D144" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="E144" t="s">
         <v>13</v>
       </c>
       <c r="F144" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G144" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="H144" t="s">
-        <v>744</v>
+        <v>10</v>
       </c>
       <c r="I144" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B145" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="C145" t="s">
         <v>10</v>
       </c>
       <c r="D145" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="E145" t="s">
         <v>13</v>
@@ -7324,10 +7594,10 @@
         <v>31</v>
       </c>
       <c r="G145" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="H145" t="s">
-        <v>749</v>
+        <v>659</v>
       </c>
       <c r="I145" t="s">
         <v>750</v>
@@ -7338,7 +7608,7 @@
         <v>751</v>
       </c>
       <c r="B146" t="s">
-        <v>718</v>
+        <v>36</v>
       </c>
       <c r="C146" t="s">
         <v>10</v>
@@ -7350,30 +7620,30 @@
         <v>13</v>
       </c>
       <c r="F146" t="s">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="G146" t="s">
         <v>753</v>
       </c>
       <c r="H146" t="s">
-        <v>721</v>
+        <v>754</v>
       </c>
       <c r="I146" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="B147" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C147" t="s">
         <v>10</v>
       </c>
       <c r="D147" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="E147" t="s">
         <v>13</v>
@@ -7382,18 +7652,18 @@
         <v>31</v>
       </c>
       <c r="G147" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="H147" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="I147" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="B148" t="s">
         <v>84</v>
@@ -7402,7 +7672,7 @@
         <v>10</v>
       </c>
       <c r="D148" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="E148" t="s">
         <v>13</v>
@@ -7411,97 +7681,97 @@
         <v>31</v>
       </c>
       <c r="G148" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="H148" t="s">
-        <v>726</v>
+        <v>764</v>
       </c>
       <c r="I148" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="B149" t="s">
-        <v>10</v>
+        <v>733</v>
       </c>
       <c r="C149" t="s">
-        <v>713</v>
+        <v>10</v>
       </c>
       <c r="D149" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="E149" t="s">
         <v>13</v>
       </c>
       <c r="F149" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="G149" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="H149" t="s">
-        <v>10</v>
+        <v>736</v>
       </c>
       <c r="I149" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="B150" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C150" t="s">
-        <v>713</v>
+        <v>10</v>
       </c>
       <c r="D150" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="E150" t="s">
         <v>13</v>
       </c>
       <c r="F150" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G150" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="H150" t="s">
-        <v>10</v>
+        <v>773</v>
       </c>
       <c r="I150" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="B151" t="s">
-        <v>773</v>
+        <v>84</v>
       </c>
       <c r="C151" t="s">
         <v>10</v>
       </c>
       <c r="D151" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="E151" t="s">
         <v>13</v>
       </c>
       <c r="F151" t="s">
-        <v>775</v>
+        <v>31</v>
       </c>
       <c r="G151" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="H151" t="s">
-        <v>777</v>
+        <v>741</v>
       </c>
       <c r="I151" t="s">
         <v>778</v>
@@ -7512,181 +7782,181 @@
         <v>779</v>
       </c>
       <c r="B152" t="s">
+        <v>10</v>
+      </c>
+      <c r="C152" t="s">
+        <v>728</v>
+      </c>
+      <c r="D152" t="s">
         <v>780</v>
       </c>
-      <c r="C152" t="s">
-        <v>10</v>
-      </c>
-      <c r="D152" t="s">
+      <c r="E152" t="s">
+        <v>13</v>
+      </c>
+      <c r="F152" t="s">
+        <v>14</v>
+      </c>
+      <c r="G152" t="s">
         <v>781</v>
       </c>
-      <c r="E152" t="s">
-        <v>13</v>
-      </c>
-      <c r="F152" t="s">
-        <v>116</v>
-      </c>
-      <c r="G152" t="s">
+      <c r="H152" t="s">
+        <v>10</v>
+      </c>
+      <c r="I152" t="s">
         <v>782</v>
-      </c>
-      <c r="H152" t="s">
-        <v>783</v>
-      </c>
-      <c r="I152" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
+        <v>783</v>
+      </c>
+      <c r="B153" t="s">
+        <v>84</v>
+      </c>
+      <c r="C153" t="s">
+        <v>10</v>
+      </c>
+      <c r="D153" t="s">
+        <v>784</v>
+      </c>
+      <c r="E153" t="s">
+        <v>13</v>
+      </c>
+      <c r="F153" t="s">
+        <v>31</v>
+      </c>
+      <c r="G153" t="s">
         <v>785</v>
       </c>
-      <c r="B153" t="s">
-        <v>780</v>
-      </c>
-      <c r="C153" t="s">
-        <v>10</v>
-      </c>
-      <c r="D153" t="s">
+      <c r="H153" t="s">
         <v>786</v>
       </c>
-      <c r="E153" t="s">
-        <v>13</v>
-      </c>
-      <c r="F153" t="s">
-        <v>116</v>
-      </c>
-      <c r="G153" t="s">
+      <c r="I153" t="s">
         <v>787</v>
-      </c>
-      <c r="H153" t="s">
-        <v>788</v>
-      </c>
-      <c r="I153" t="s">
-        <v>789</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
+        <v>788</v>
+      </c>
+      <c r="B154" t="s">
+        <v>10</v>
+      </c>
+      <c r="C154" t="s">
+        <v>728</v>
+      </c>
+      <c r="D154" t="s">
+        <v>789</v>
+      </c>
+      <c r="E154" t="s">
+        <v>13</v>
+      </c>
+      <c r="F154" t="s">
+        <v>14</v>
+      </c>
+      <c r="G154" t="s">
         <v>790</v>
       </c>
-      <c r="B154" t="s">
+      <c r="H154" t="s">
+        <v>10</v>
+      </c>
+      <c r="I154" t="s">
         <v>791</v>
-      </c>
-      <c r="C154" t="s">
-        <v>10</v>
-      </c>
-      <c r="D154" t="s">
-        <v>792</v>
-      </c>
-      <c r="E154" t="s">
-        <v>13</v>
-      </c>
-      <c r="F154" t="s">
-        <v>793</v>
-      </c>
-      <c r="G154" t="s">
-        <v>794</v>
-      </c>
-      <c r="H154" t="s">
-        <v>10</v>
-      </c>
-      <c r="I154" t="s">
-        <v>795</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
+        <v>792</v>
+      </c>
+      <c r="B155" t="s">
+        <v>793</v>
+      </c>
+      <c r="C155" t="s">
+        <v>10</v>
+      </c>
+      <c r="D155" t="s">
+        <v>794</v>
+      </c>
+      <c r="E155" t="s">
+        <v>13</v>
+      </c>
+      <c r="F155" t="s">
+        <v>795</v>
+      </c>
+      <c r="G155" t="s">
         <v>796</v>
       </c>
-      <c r="B155" t="s">
-        <v>36</v>
-      </c>
-      <c r="C155" t="s">
-        <v>10</v>
-      </c>
-      <c r="D155" t="s">
+      <c r="H155" t="s">
         <v>797</v>
       </c>
-      <c r="E155" t="s">
-        <v>13</v>
-      </c>
-      <c r="F155" t="s">
-        <v>31</v>
-      </c>
-      <c r="G155" t="s">
+      <c r="I155" t="s">
         <v>798</v>
-      </c>
-      <c r="H155" t="s">
-        <v>799</v>
-      </c>
-      <c r="I155" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
+        <v>799</v>
+      </c>
+      <c r="B156" t="s">
+        <v>800</v>
+      </c>
+      <c r="C156" t="s">
+        <v>10</v>
+      </c>
+      <c r="D156" t="s">
         <v>801</v>
       </c>
-      <c r="B156" t="s">
-        <v>90</v>
-      </c>
-      <c r="C156" t="s">
-        <v>10</v>
-      </c>
-      <c r="D156" t="s">
+      <c r="E156" t="s">
+        <v>13</v>
+      </c>
+      <c r="F156" t="s">
+        <v>116</v>
+      </c>
+      <c r="G156" t="s">
         <v>802</v>
       </c>
-      <c r="E156" t="s">
-        <v>13</v>
-      </c>
-      <c r="F156" t="s">
-        <v>31</v>
-      </c>
-      <c r="G156" t="s">
+      <c r="H156" t="s">
         <v>803</v>
       </c>
-      <c r="H156" t="s">
+      <c r="I156" t="s">
         <v>804</v>
-      </c>
-      <c r="I156" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
+        <v>805</v>
+      </c>
+      <c r="B157" t="s">
+        <v>800</v>
+      </c>
+      <c r="C157" t="s">
+        <v>10</v>
+      </c>
+      <c r="D157" t="s">
         <v>806</v>
       </c>
-      <c r="B157" t="s">
-        <v>36</v>
-      </c>
-      <c r="C157" t="s">
-        <v>10</v>
-      </c>
-      <c r="D157" t="s">
+      <c r="E157" t="s">
+        <v>13</v>
+      </c>
+      <c r="F157" t="s">
+        <v>116</v>
+      </c>
+      <c r="G157" t="s">
         <v>807</v>
       </c>
-      <c r="E157" t="s">
-        <v>13</v>
-      </c>
-      <c r="F157" t="s">
-        <v>31</v>
-      </c>
-      <c r="G157" t="s">
+      <c r="H157" t="s">
         <v>808</v>
       </c>
-      <c r="H157" t="s">
+      <c r="I157" t="s">
         <v>809</v>
-      </c>
-      <c r="I157" t="s">
-        <v>810</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
+        <v>810</v>
+      </c>
+      <c r="B158" t="s">
         <v>811</v>
-      </c>
-      <c r="B158" t="s">
-        <v>36</v>
       </c>
       <c r="C158" t="s">
         <v>10</v>
@@ -7698,13 +7968,13 @@
         <v>13</v>
       </c>
       <c r="F158" t="s">
-        <v>31</v>
+        <v>813</v>
       </c>
       <c r="G158" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="H158" t="s">
-        <v>814</v>
+        <v>10</v>
       </c>
       <c r="I158" t="s">
         <v>815</v>
@@ -7715,7 +7985,7 @@
         <v>816</v>
       </c>
       <c r="B159" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="C159" t="s">
         <v>10</v>
@@ -7744,123 +8014,123 @@
         <v>821</v>
       </c>
       <c r="B160" t="s">
+        <v>90</v>
+      </c>
+      <c r="C160" t="s">
+        <v>10</v>
+      </c>
+      <c r="D160" t="s">
         <v>822</v>
       </c>
-      <c r="C160" t="s">
-        <v>10</v>
-      </c>
-      <c r="D160" t="s">
+      <c r="E160" t="s">
+        <v>13</v>
+      </c>
+      <c r="F160" t="s">
+        <v>31</v>
+      </c>
+      <c r="G160" t="s">
         <v>823</v>
       </c>
-      <c r="E160" t="s">
-        <v>13</v>
-      </c>
-      <c r="F160" t="s">
-        <v>31</v>
-      </c>
-      <c r="G160" t="s">
+      <c r="H160" t="s">
         <v>824</v>
       </c>
-      <c r="H160" t="s">
+      <c r="I160" t="s">
         <v>825</v>
-      </c>
-      <c r="I160" t="s">
-        <v>826</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
+        <v>826</v>
+      </c>
+      <c r="B161" t="s">
+        <v>36</v>
+      </c>
+      <c r="C161" t="s">
+        <v>10</v>
+      </c>
+      <c r="D161" t="s">
         <v>827</v>
       </c>
-      <c r="B161" t="s">
-        <v>84</v>
-      </c>
-      <c r="C161" t="s">
-        <v>10</v>
-      </c>
-      <c r="D161" t="s">
+      <c r="E161" t="s">
+        <v>13</v>
+      </c>
+      <c r="F161" t="s">
+        <v>31</v>
+      </c>
+      <c r="G161" t="s">
         <v>828</v>
       </c>
-      <c r="E161" t="s">
-        <v>13</v>
-      </c>
-      <c r="F161" t="s">
-        <v>31</v>
-      </c>
-      <c r="G161" t="s">
+      <c r="H161" t="s">
         <v>829</v>
       </c>
-      <c r="H161" t="s">
+      <c r="I161" t="s">
         <v>830</v>
-      </c>
-      <c r="I161" t="s">
-        <v>831</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
+        <v>831</v>
+      </c>
+      <c r="B162" t="s">
+        <v>36</v>
+      </c>
+      <c r="C162" t="s">
+        <v>10</v>
+      </c>
+      <c r="D162" t="s">
         <v>832</v>
       </c>
-      <c r="B162" t="s">
-        <v>84</v>
-      </c>
-      <c r="C162" t="s">
-        <v>10</v>
-      </c>
-      <c r="D162" t="s">
+      <c r="E162" t="s">
+        <v>13</v>
+      </c>
+      <c r="F162" t="s">
+        <v>31</v>
+      </c>
+      <c r="G162" t="s">
         <v>833</v>
       </c>
-      <c r="E162" t="s">
-        <v>13</v>
-      </c>
-      <c r="F162" t="s">
-        <v>31</v>
-      </c>
-      <c r="G162" t="s">
+      <c r="H162" t="s">
         <v>834</v>
       </c>
-      <c r="H162" t="s">
+      <c r="I162" t="s">
         <v>835</v>
-      </c>
-      <c r="I162" t="s">
-        <v>836</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
+        <v>836</v>
+      </c>
+      <c r="B163" t="s">
+        <v>84</v>
+      </c>
+      <c r="C163" t="s">
+        <v>10</v>
+      </c>
+      <c r="D163" t="s">
         <v>837</v>
       </c>
-      <c r="B163" t="s">
-        <v>36</v>
-      </c>
-      <c r="C163" t="s">
-        <v>10</v>
-      </c>
-      <c r="D163" t="s">
+      <c r="E163" t="s">
+        <v>13</v>
+      </c>
+      <c r="F163" t="s">
+        <v>31</v>
+      </c>
+      <c r="G163" t="s">
         <v>838</v>
       </c>
-      <c r="E163" t="s">
-        <v>13</v>
-      </c>
-      <c r="F163" t="s">
-        <v>31</v>
-      </c>
-      <c r="G163" t="s">
+      <c r="H163" t="s">
         <v>839</v>
       </c>
-      <c r="H163" t="s">
+      <c r="I163" t="s">
         <v>840</v>
-      </c>
-      <c r="I163" t="s">
-        <v>841</v>
       </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
+        <v>841</v>
+      </c>
+      <c r="B164" t="s">
         <v>842</v>
-      </c>
-      <c r="B164" t="s">
-        <v>36</v>
       </c>
       <c r="C164" t="s">
         <v>10</v>
@@ -7918,7 +8188,7 @@
         <v>852</v>
       </c>
       <c r="B166" t="s">
-        <v>237</v>
+        <v>84</v>
       </c>
       <c r="C166" t="s">
         <v>10</v>
@@ -7947,7 +8217,7 @@
         <v>857</v>
       </c>
       <c r="B167" t="s">
-        <v>195</v>
+        <v>36</v>
       </c>
       <c r="C167" t="s">
         <v>10</v>
@@ -8034,7 +8304,7 @@
         <v>872</v>
       </c>
       <c r="B170" t="s">
-        <v>36</v>
+        <v>237</v>
       </c>
       <c r="C170" t="s">
         <v>10</v>
@@ -8063,7 +8333,7 @@
         <v>877</v>
       </c>
       <c r="B171" t="s">
-        <v>84</v>
+        <v>195</v>
       </c>
       <c r="C171" t="s">
         <v>10</v>
@@ -8092,33 +8362,33 @@
         <v>882</v>
       </c>
       <c r="B172" t="s">
+        <v>36</v>
+      </c>
+      <c r="C172" t="s">
+        <v>10</v>
+      </c>
+      <c r="D172" t="s">
         <v>883</v>
       </c>
-      <c r="C172" t="s">
-        <v>10</v>
-      </c>
-      <c r="D172" t="s">
+      <c r="E172" t="s">
+        <v>13</v>
+      </c>
+      <c r="F172" t="s">
+        <v>31</v>
+      </c>
+      <c r="G172" t="s">
         <v>884</v>
       </c>
-      <c r="E172" t="s">
-        <v>13</v>
-      </c>
-      <c r="F172" t="s">
-        <v>31</v>
-      </c>
-      <c r="G172" t="s">
+      <c r="H172" t="s">
         <v>885</v>
       </c>
-      <c r="H172" t="s">
+      <c r="I172" t="s">
         <v>886</v>
-      </c>
-      <c r="I172" t="s">
-        <v>887</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B173" t="s">
         <v>84</v>
@@ -8127,80 +8397,602 @@
         <v>10</v>
       </c>
       <c r="D173" t="s">
+        <v>888</v>
+      </c>
+      <c r="E173" t="s">
+        <v>13</v>
+      </c>
+      <c r="F173" t="s">
+        <v>31</v>
+      </c>
+      <c r="G173" t="s">
         <v>889</v>
       </c>
-      <c r="E173" t="s">
-        <v>13</v>
-      </c>
-      <c r="F173" t="s">
-        <v>31</v>
-      </c>
-      <c r="G173" t="s">
+      <c r="H173" t="s">
         <v>890</v>
       </c>
-      <c r="H173" t="s">
+      <c r="I173" t="s">
         <v>891</v>
-      </c>
-      <c r="I173" t="s">
-        <v>892</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>892</v>
+      </c>
+      <c r="B174" t="s">
+        <v>36</v>
+      </c>
+      <c r="C174" t="s">
+        <v>10</v>
+      </c>
+      <c r="D174" t="s">
         <v>893</v>
       </c>
-      <c r="B174" t="s">
+      <c r="E174" t="s">
+        <v>13</v>
+      </c>
+      <c r="F174" t="s">
+        <v>31</v>
+      </c>
+      <c r="G174" t="s">
         <v>894</v>
       </c>
-      <c r="C174" t="s">
-        <v>10</v>
-      </c>
-      <c r="D174" t="s">
+      <c r="H174" t="s">
         <v>895</v>
       </c>
-      <c r="E174" t="s">
-        <v>13</v>
-      </c>
-      <c r="F174" t="s">
-        <v>775</v>
-      </c>
-      <c r="G174" t="s">
+      <c r="I174" t="s">
         <v>896</v>
-      </c>
-      <c r="H174" t="s">
-        <v>897</v>
-      </c>
-      <c r="I174" t="s">
-        <v>898</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
+        <v>897</v>
+      </c>
+      <c r="B175" t="s">
+        <v>84</v>
+      </c>
+      <c r="C175" t="s">
+        <v>10</v>
+      </c>
+      <c r="D175" t="s">
+        <v>898</v>
+      </c>
+      <c r="E175" t="s">
+        <v>13</v>
+      </c>
+      <c r="F175" t="s">
+        <v>31</v>
+      </c>
+      <c r="G175" t="s">
         <v>899</v>
       </c>
-      <c r="B175" t="s">
+      <c r="H175" t="s">
         <v>900</v>
       </c>
-      <c r="C175" t="s">
-        <v>10</v>
-      </c>
-      <c r="D175" t="s">
+      <c r="I175" t="s">
         <v>901</v>
       </c>
-      <c r="E175" t="s">
-        <v>13</v>
-      </c>
-      <c r="F175" t="s">
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
         <v>902</v>
       </c>
-      <c r="G175" t="s">
+      <c r="B176" t="s">
+        <v>29</v>
+      </c>
+      <c r="C176" t="s">
+        <v>10</v>
+      </c>
+      <c r="D176" t="s">
         <v>903</v>
       </c>
-      <c r="H175" t="s">
+      <c r="E176" t="s">
+        <v>13</v>
+      </c>
+      <c r="F176" t="s">
+        <v>31</v>
+      </c>
+      <c r="G176" t="s">
         <v>904</v>
       </c>
-      <c r="I175" t="s">
+      <c r="H176" t="s">
         <v>905</v>
+      </c>
+      <c r="I176" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>907</v>
+      </c>
+      <c r="B177" t="s">
+        <v>36</v>
+      </c>
+      <c r="C177" t="s">
+        <v>10</v>
+      </c>
+      <c r="D177" t="s">
+        <v>908</v>
+      </c>
+      <c r="E177" t="s">
+        <v>13</v>
+      </c>
+      <c r="F177" t="s">
+        <v>31</v>
+      </c>
+      <c r="G177" t="s">
+        <v>909</v>
+      </c>
+      <c r="H177" t="s">
+        <v>910</v>
+      </c>
+      <c r="I177" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>912</v>
+      </c>
+      <c r="B178" t="s">
+        <v>36</v>
+      </c>
+      <c r="C178" t="s">
+        <v>10</v>
+      </c>
+      <c r="D178" t="s">
+        <v>913</v>
+      </c>
+      <c r="E178" t="s">
+        <v>13</v>
+      </c>
+      <c r="F178" t="s">
+        <v>31</v>
+      </c>
+      <c r="G178" t="s">
+        <v>914</v>
+      </c>
+      <c r="H178" t="s">
+        <v>915</v>
+      </c>
+      <c r="I178" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>917</v>
+      </c>
+      <c r="B179" t="s">
+        <v>36</v>
+      </c>
+      <c r="C179" t="s">
+        <v>10</v>
+      </c>
+      <c r="D179" t="s">
+        <v>918</v>
+      </c>
+      <c r="E179" t="s">
+        <v>13</v>
+      </c>
+      <c r="F179" t="s">
+        <v>31</v>
+      </c>
+      <c r="G179" t="s">
+        <v>919</v>
+      </c>
+      <c r="H179" t="s">
+        <v>920</v>
+      </c>
+      <c r="I179" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>922</v>
+      </c>
+      <c r="B180" t="s">
+        <v>90</v>
+      </c>
+      <c r="C180" t="s">
+        <v>10</v>
+      </c>
+      <c r="D180" t="s">
+        <v>923</v>
+      </c>
+      <c r="E180" t="s">
+        <v>13</v>
+      </c>
+      <c r="F180" t="s">
+        <v>31</v>
+      </c>
+      <c r="G180" t="s">
+        <v>924</v>
+      </c>
+      <c r="H180" t="s">
+        <v>925</v>
+      </c>
+      <c r="I180" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>927</v>
+      </c>
+      <c r="B181" t="s">
+        <v>84</v>
+      </c>
+      <c r="C181" t="s">
+        <v>10</v>
+      </c>
+      <c r="D181" t="s">
+        <v>928</v>
+      </c>
+      <c r="E181" t="s">
+        <v>13</v>
+      </c>
+      <c r="F181" t="s">
+        <v>31</v>
+      </c>
+      <c r="G181" t="s">
+        <v>929</v>
+      </c>
+      <c r="H181" t="s">
+        <v>930</v>
+      </c>
+      <c r="I181" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>932</v>
+      </c>
+      <c r="B182" t="s">
+        <v>933</v>
+      </c>
+      <c r="C182" t="s">
+        <v>10</v>
+      </c>
+      <c r="D182" t="s">
+        <v>934</v>
+      </c>
+      <c r="E182" t="s">
+        <v>13</v>
+      </c>
+      <c r="F182" t="s">
+        <v>31</v>
+      </c>
+      <c r="G182" t="s">
+        <v>935</v>
+      </c>
+      <c r="H182" t="s">
+        <v>936</v>
+      </c>
+      <c r="I182" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>938</v>
+      </c>
+      <c r="B183" t="s">
+        <v>84</v>
+      </c>
+      <c r="C183" t="s">
+        <v>10</v>
+      </c>
+      <c r="D183" t="s">
+        <v>939</v>
+      </c>
+      <c r="E183" t="s">
+        <v>13</v>
+      </c>
+      <c r="F183" t="s">
+        <v>31</v>
+      </c>
+      <c r="G183" t="s">
+        <v>940</v>
+      </c>
+      <c r="H183" t="s">
+        <v>941</v>
+      </c>
+      <c r="I183" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>943</v>
+      </c>
+      <c r="B184" t="s">
+        <v>36</v>
+      </c>
+      <c r="C184" t="s">
+        <v>10</v>
+      </c>
+      <c r="D184" t="s">
+        <v>944</v>
+      </c>
+      <c r="E184" t="s">
+        <v>13</v>
+      </c>
+      <c r="F184" t="s">
+        <v>31</v>
+      </c>
+      <c r="G184" t="s">
+        <v>945</v>
+      </c>
+      <c r="H184" t="s">
+        <v>946</v>
+      </c>
+      <c r="I184" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>948</v>
+      </c>
+      <c r="B185" t="s">
+        <v>933</v>
+      </c>
+      <c r="C185" t="s">
+        <v>10</v>
+      </c>
+      <c r="D185" t="s">
+        <v>949</v>
+      </c>
+      <c r="E185" t="s">
+        <v>13</v>
+      </c>
+      <c r="F185" t="s">
+        <v>31</v>
+      </c>
+      <c r="G185" t="s">
+        <v>950</v>
+      </c>
+      <c r="H185" t="s">
+        <v>951</v>
+      </c>
+      <c r="I185" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>953</v>
+      </c>
+      <c r="B186" t="s">
+        <v>195</v>
+      </c>
+      <c r="C186" t="s">
+        <v>10</v>
+      </c>
+      <c r="D186" t="s">
+        <v>954</v>
+      </c>
+      <c r="E186" t="s">
+        <v>13</v>
+      </c>
+      <c r="F186" t="s">
+        <v>31</v>
+      </c>
+      <c r="G186" t="s">
+        <v>955</v>
+      </c>
+      <c r="H186" t="s">
+        <v>956</v>
+      </c>
+      <c r="I186" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>958</v>
+      </c>
+      <c r="B187" t="s">
+        <v>29</v>
+      </c>
+      <c r="C187" t="s">
+        <v>10</v>
+      </c>
+      <c r="D187" t="s">
+        <v>959</v>
+      </c>
+      <c r="E187" t="s">
+        <v>13</v>
+      </c>
+      <c r="F187" t="s">
+        <v>31</v>
+      </c>
+      <c r="G187" t="s">
+        <v>960</v>
+      </c>
+      <c r="H187" t="s">
+        <v>961</v>
+      </c>
+      <c r="I187" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>963</v>
+      </c>
+      <c r="B188" t="s">
+        <v>36</v>
+      </c>
+      <c r="C188" t="s">
+        <v>10</v>
+      </c>
+      <c r="D188" t="s">
+        <v>964</v>
+      </c>
+      <c r="E188" t="s">
+        <v>13</v>
+      </c>
+      <c r="F188" t="s">
+        <v>31</v>
+      </c>
+      <c r="G188" t="s">
+        <v>965</v>
+      </c>
+      <c r="H188" t="s">
+        <v>966</v>
+      </c>
+      <c r="I188" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>968</v>
+      </c>
+      <c r="B189" t="s">
+        <v>36</v>
+      </c>
+      <c r="C189" t="s">
+        <v>10</v>
+      </c>
+      <c r="D189" t="s">
+        <v>969</v>
+      </c>
+      <c r="E189" t="s">
+        <v>13</v>
+      </c>
+      <c r="F189" t="s">
+        <v>31</v>
+      </c>
+      <c r="G189" t="s">
+        <v>970</v>
+      </c>
+      <c r="H189" t="s">
+        <v>971</v>
+      </c>
+      <c r="I189" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>973</v>
+      </c>
+      <c r="B190" t="s">
+        <v>36</v>
+      </c>
+      <c r="C190" t="s">
+        <v>10</v>
+      </c>
+      <c r="D190" t="s">
+        <v>974</v>
+      </c>
+      <c r="E190" t="s">
+        <v>13</v>
+      </c>
+      <c r="F190" t="s">
+        <v>31</v>
+      </c>
+      <c r="G190" t="s">
+        <v>975</v>
+      </c>
+      <c r="H190" t="s">
+        <v>976</v>
+      </c>
+      <c r="I190" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>978</v>
+      </c>
+      <c r="B191" t="s">
+        <v>36</v>
+      </c>
+      <c r="C191" t="s">
+        <v>10</v>
+      </c>
+      <c r="D191" t="s">
+        <v>979</v>
+      </c>
+      <c r="E191" t="s">
+        <v>13</v>
+      </c>
+      <c r="F191" t="s">
+        <v>31</v>
+      </c>
+      <c r="G191" t="s">
+        <v>980</v>
+      </c>
+      <c r="H191" t="s">
+        <v>981</v>
+      </c>
+      <c r="I191" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>983</v>
+      </c>
+      <c r="B192" t="s">
+        <v>984</v>
+      </c>
+      <c r="C192" t="s">
+        <v>10</v>
+      </c>
+      <c r="D192" t="s">
+        <v>985</v>
+      </c>
+      <c r="E192" t="s">
+        <v>13</v>
+      </c>
+      <c r="F192" t="s">
+        <v>795</v>
+      </c>
+      <c r="G192" t="s">
+        <v>986</v>
+      </c>
+      <c r="H192" t="s">
+        <v>987</v>
+      </c>
+      <c r="I192" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>989</v>
+      </c>
+      <c r="B193" t="s">
+        <v>990</v>
+      </c>
+      <c r="C193" t="s">
+        <v>10</v>
+      </c>
+      <c r="D193" t="s">
+        <v>991</v>
+      </c>
+      <c r="E193" t="s">
+        <v>13</v>
+      </c>
+      <c r="F193" t="s">
+        <v>992</v>
+      </c>
+      <c r="G193" t="s">
+        <v>993</v>
+      </c>
+      <c r="H193" t="s">
+        <v>994</v>
+      </c>
+      <c r="I193" t="s">
+        <v>995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(import): state of the last homepage and current travel information re-import and upload (progress, upload state, reports, url lists)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -1267,7 +1267,7 @@
     <t>at/de/homepage.report.json</t>
   </si>
   <si>
-    <t>["flight-search","hero-card-overlay","fare-teaser","carousel-cards","destination-finder","cards-icon","columns-logos","accordion-columns"]</t>
+    <t>["flash-teaser","flight-search","hero-card-overlay","fare-teaser","carousel-cards","destination-finder","cards-icon","columns-logos","accordion-columns"]</t>
   </si>
   <si>
     <t>at/de/homepage</t>
@@ -1276,7 +1276,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-25T08:30:46.785Z</t>
+    <t>2026-10-25T08:54:33.653Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/homepage</t>
@@ -3652,7 +3652,7 @@
     <t>de/de/homepage</t>
   </si>
   <si>
-    <t>2026-10-25T05:34:40.233Z</t>
+    <t>2026-10-25T08:54:30.620Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/homepage</t>
@@ -5965,7 +5965,7 @@
     <t>de/en/homepage</t>
   </si>
   <si>
-    <t>2026-10-25T05:34:37.272Z</t>
+    <t>2026-10-25T08:54:26.667Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/homepage</t>
@@ -8227,7 +8227,7 @@
     <t>gb/en/homepage</t>
   </si>
   <si>
-    <t>2026-10-25T05:34:47.202Z</t>
+    <t>2026-10-25T08:54:36.437Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/homepage</t>

</xml_diff>